<commit_message>
UI Tram Dien TKVV
</commit_message>
<xml_diff>
--- a/public/TagWarning.xlsx
+++ b/public/TagWarning.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24131"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DC1A414-8552-41C5-A457-78280B3DB240}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83EE638B-6596-4206-9343-90256256D219}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="10" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="10" activeTab="16" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LBMT_PLDM#1" sheetId="1" r:id="rId1"/>
@@ -1625,9 +1625,6 @@
     <t>VI822bM</t>
   </si>
   <si>
-    <t>CT-HF2</t>
-  </si>
-  <si>
     <t>TI835aM</t>
   </si>
   <si>
@@ -1652,9 +1649,6 @@
     <t>VI831bM</t>
   </si>
   <si>
-    <t>CT-HF3</t>
-  </si>
-  <si>
     <t>TI845aM</t>
   </si>
   <si>
@@ -1676,9 +1670,6 @@
     <t>VI842aM</t>
   </si>
   <si>
-    <t>CT-HF4</t>
-  </si>
-  <si>
     <t>TI814M</t>
   </si>
   <si>
@@ -1773,6 +1764,15 @@
   </si>
   <si>
     <t>VI843bM</t>
+  </si>
+  <si>
+    <t>CT_HF2</t>
+  </si>
+  <si>
+    <t>CT_HF3</t>
+  </si>
+  <si>
+    <t>CT_HF4</t>
   </si>
 </sst>
 </file>
@@ -2270,10 +2270,10 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2984,6 +2984,12 @@
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="B1:D1"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="B4:D4"/>
     <mergeCell ref="B16:D16"/>
     <mergeCell ref="B15:D15"/>
     <mergeCell ref="B14:D14"/>
@@ -2994,12 +3000,6 @@
     <mergeCell ref="B11:D11"/>
     <mergeCell ref="B10:D10"/>
     <mergeCell ref="B9:D9"/>
-    <mergeCell ref="B1:D1"/>
-    <mergeCell ref="B5:D5"/>
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="B7:D7"/>
-    <mergeCell ref="B6:D6"/>
-    <mergeCell ref="B4:D4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="261" orientation="landscape" horizontalDpi="180" verticalDpi="180" r:id="rId1"/>
@@ -3360,6 +3360,13 @@
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="A10:C10"/>
+    <mergeCell ref="A9:C9"/>
+    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="A14:C14"/>
+    <mergeCell ref="A13:C13"/>
+    <mergeCell ref="A12:C12"/>
+    <mergeCell ref="A11:C11"/>
     <mergeCell ref="A3:C3"/>
     <mergeCell ref="A2:C2"/>
     <mergeCell ref="A1:C1"/>
@@ -3368,13 +3375,6 @@
     <mergeCell ref="A6:C6"/>
     <mergeCell ref="A5:C5"/>
     <mergeCell ref="A4:C4"/>
-    <mergeCell ref="A10:C10"/>
-    <mergeCell ref="A9:C9"/>
-    <mergeCell ref="A15:C15"/>
-    <mergeCell ref="A14:C14"/>
-    <mergeCell ref="A13:C13"/>
-    <mergeCell ref="A12:C12"/>
-    <mergeCell ref="A11:C11"/>
   </mergeCells>
   <phoneticPr fontId="12" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3765,6 +3765,13 @@
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="A7:C7"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="A5:C5"/>
     <mergeCell ref="A13:C13"/>
     <mergeCell ref="A14:C14"/>
     <mergeCell ref="A15:C15"/>
@@ -3773,13 +3780,6 @@
     <mergeCell ref="A10:C10"/>
     <mergeCell ref="A11:C11"/>
     <mergeCell ref="A12:C12"/>
-    <mergeCell ref="A6:C6"/>
-    <mergeCell ref="A7:C7"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="A3:C3"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="A5:C5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4140,6 +4140,13 @@
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="A7:C7"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="A5:C5"/>
     <mergeCell ref="A13:C13"/>
     <mergeCell ref="A14:C14"/>
     <mergeCell ref="A15:C15"/>
@@ -4148,13 +4155,6 @@
     <mergeCell ref="A10:C10"/>
     <mergeCell ref="A11:C11"/>
     <mergeCell ref="A12:C12"/>
-    <mergeCell ref="A6:C6"/>
-    <mergeCell ref="A7:C7"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="A3:C3"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="A5:C5"/>
   </mergeCells>
   <phoneticPr fontId="12" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -8526,13 +8526,13 @@
         <v>223</v>
       </c>
       <c r="B1" s="41" t="s">
-        <v>558</v>
+        <v>555</v>
       </c>
       <c r="C1" s="42" t="s">
         <v>0</v>
       </c>
       <c r="D1" s="38" t="s">
-        <v>568</v>
+        <v>565</v>
       </c>
       <c r="E1" s="38" t="s">
         <v>33</v>
@@ -8549,13 +8549,13 @@
         <v>223</v>
       </c>
       <c r="B2" s="41" t="s">
-        <v>559</v>
+        <v>556</v>
       </c>
       <c r="C2" s="46" t="s">
         <v>1</v>
       </c>
       <c r="D2" s="38" t="s">
-        <v>569</v>
+        <v>566</v>
       </c>
       <c r="E2" s="47" t="s">
         <v>33</v>
@@ -8572,13 +8572,13 @@
         <v>223</v>
       </c>
       <c r="B3" s="41" t="s">
-        <v>560</v>
+        <v>557</v>
       </c>
       <c r="C3" s="46" t="s">
         <v>3</v>
       </c>
       <c r="D3" s="38" t="s">
-        <v>570</v>
+        <v>567</v>
       </c>
       <c r="E3" s="47" t="s">
         <v>33</v>
@@ -8601,7 +8601,7 @@
         <v>5</v>
       </c>
       <c r="D4" s="38" t="s">
-        <v>547</v>
+        <v>544</v>
       </c>
       <c r="E4" s="47" t="s">
         <v>33</v>
@@ -8618,7 +8618,7 @@
         <v>223</v>
       </c>
       <c r="B5" s="45" t="s">
-        <v>557</v>
+        <v>554</v>
       </c>
       <c r="C5" s="46" t="s">
         <v>7</v>
@@ -8641,7 +8641,7 @@
         <v>223</v>
       </c>
       <c r="B6" s="45" t="s">
-        <v>561</v>
+        <v>558</v>
       </c>
       <c r="C6" s="46" t="s">
         <v>9</v>
@@ -8687,13 +8687,13 @@
         <v>223</v>
       </c>
       <c r="B8" s="45" t="s">
-        <v>562</v>
+        <v>559</v>
       </c>
       <c r="C8" s="46" t="s">
         <v>14</v>
       </c>
       <c r="D8" s="52" t="s">
-        <v>571</v>
+        <v>568</v>
       </c>
       <c r="E8" s="47" t="s">
         <v>67</v>
@@ -8716,7 +8716,7 @@
         <v>16</v>
       </c>
       <c r="D9" s="52" t="s">
-        <v>572</v>
+        <v>569</v>
       </c>
       <c r="E9" s="47" t="s">
         <v>67</v>
@@ -8733,7 +8733,7 @@
         <v>223</v>
       </c>
       <c r="B10" s="45" t="s">
-        <v>563</v>
+        <v>560</v>
       </c>
       <c r="C10" s="46" t="s">
         <v>18</v>
@@ -8756,7 +8756,7 @@
         <v>223</v>
       </c>
       <c r="B11" s="45" t="s">
-        <v>564</v>
+        <v>561</v>
       </c>
       <c r="C11" s="46" t="s">
         <v>19</v>
@@ -8779,7 +8779,7 @@
         <v>223</v>
       </c>
       <c r="B12" s="45" t="s">
-        <v>565</v>
+        <v>562</v>
       </c>
       <c r="C12" s="46" t="s">
         <v>20</v>
@@ -8802,7 +8802,7 @@
         <v>223</v>
       </c>
       <c r="B13" s="45" t="s">
-        <v>566</v>
+        <v>563</v>
       </c>
       <c r="C13" s="46" t="s">
         <v>21</v>
@@ -8844,7 +8844,7 @@
         <v>273</v>
       </c>
       <c r="B15" s="41" t="s">
-        <v>558</v>
+        <v>555</v>
       </c>
       <c r="C15" s="46" t="s">
         <v>23</v>
@@ -8867,7 +8867,7 @@
         <v>273</v>
       </c>
       <c r="B16" s="41" t="s">
-        <v>559</v>
+        <v>556</v>
       </c>
       <c r="C16" s="46" t="s">
         <v>24</v>
@@ -8890,7 +8890,7 @@
         <v>273</v>
       </c>
       <c r="B17" s="41" t="s">
-        <v>560</v>
+        <v>557</v>
       </c>
       <c r="C17" s="46" t="s">
         <v>112</v>
@@ -8936,13 +8936,13 @@
         <v>273</v>
       </c>
       <c r="B19" s="51" t="s">
-        <v>557</v>
+        <v>554</v>
       </c>
       <c r="C19" s="46" t="s">
         <v>114</v>
       </c>
       <c r="D19" s="53" t="s">
-        <v>550</v>
+        <v>547</v>
       </c>
       <c r="E19" s="47" t="s">
         <v>33</v>
@@ -8959,13 +8959,13 @@
         <v>273</v>
       </c>
       <c r="B20" s="51" t="s">
-        <v>561</v>
+        <v>558</v>
       </c>
       <c r="C20" s="46" t="s">
         <v>115</v>
       </c>
       <c r="D20" s="53" t="s">
-        <v>549</v>
+        <v>546</v>
       </c>
       <c r="E20" s="47" t="s">
         <v>33</v>
@@ -8988,7 +8988,7 @@
         <v>117</v>
       </c>
       <c r="D21" s="53" t="s">
-        <v>548</v>
+        <v>545</v>
       </c>
       <c r="E21" s="47" t="s">
         <v>33</v>
@@ -9005,13 +9005,13 @@
         <v>273</v>
       </c>
       <c r="B22" s="45" t="s">
-        <v>562</v>
+        <v>559</v>
       </c>
       <c r="C22" s="46" t="s">
         <v>119</v>
       </c>
       <c r="D22" s="52" t="s">
-        <v>573</v>
+        <v>570</v>
       </c>
       <c r="E22" s="47" t="s">
         <v>67</v>
@@ -9034,7 +9034,7 @@
         <v>121</v>
       </c>
       <c r="D23" s="52" t="s">
-        <v>574</v>
+        <v>571</v>
       </c>
       <c r="E23" s="47" t="s">
         <v>67</v>
@@ -9051,7 +9051,7 @@
         <v>273</v>
       </c>
       <c r="B24" s="45" t="s">
-        <v>563</v>
+        <v>560</v>
       </c>
       <c r="C24" s="46" t="s">
         <v>123</v>
@@ -9074,7 +9074,7 @@
         <v>273</v>
       </c>
       <c r="B25" s="45" t="s">
-        <v>564</v>
+        <v>561</v>
       </c>
       <c r="C25" s="46" t="s">
         <v>348</v>
@@ -9097,7 +9097,7 @@
         <v>273</v>
       </c>
       <c r="B26" s="45" t="s">
-        <v>565</v>
+        <v>562</v>
       </c>
       <c r="C26" s="46" t="s">
         <v>349</v>
@@ -9120,7 +9120,7 @@
         <v>273</v>
       </c>
       <c r="B27" s="45" t="s">
-        <v>566</v>
+        <v>563</v>
       </c>
       <c r="C27" s="46" t="s">
         <v>350</v>
@@ -9149,7 +9149,7 @@
         <v>351</v>
       </c>
       <c r="D28" s="38" t="s">
-        <v>529</v>
+        <v>576</v>
       </c>
       <c r="E28" s="49" t="s">
         <v>402</v>
@@ -9162,13 +9162,13 @@
         <v>274</v>
       </c>
       <c r="B29" s="41" t="s">
-        <v>558</v>
+        <v>555</v>
       </c>
       <c r="C29" s="46" t="s">
         <v>352</v>
       </c>
       <c r="D29" s="38" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="E29" s="47" t="s">
         <v>33</v>
@@ -9185,13 +9185,13 @@
         <v>274</v>
       </c>
       <c r="B30" s="41" t="s">
-        <v>559</v>
+        <v>556</v>
       </c>
       <c r="C30" s="46" t="s">
         <v>353</v>
       </c>
       <c r="D30" s="38" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="E30" s="47" t="s">
         <v>33</v>
@@ -9208,13 +9208,13 @@
         <v>274</v>
       </c>
       <c r="B31" s="41" t="s">
-        <v>560</v>
+        <v>557</v>
       </c>
       <c r="C31" s="46" t="s">
         <v>354</v>
       </c>
       <c r="D31" s="38" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="E31" s="47" t="s">
         <v>33</v>
@@ -9237,7 +9237,7 @@
         <v>355</v>
       </c>
       <c r="D32" s="38" t="s">
-        <v>553</v>
+        <v>550</v>
       </c>
       <c r="E32" s="47" t="s">
         <v>33</v>
@@ -9254,13 +9254,13 @@
         <v>274</v>
       </c>
       <c r="B33" s="41" t="s">
-        <v>557</v>
+        <v>554</v>
       </c>
       <c r="C33" s="46" t="s">
         <v>356</v>
       </c>
       <c r="D33" s="38" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="E33" s="47" t="s">
         <v>33</v>
@@ -9277,13 +9277,13 @@
         <v>274</v>
       </c>
       <c r="B34" s="45" t="s">
-        <v>561</v>
+        <v>558</v>
       </c>
       <c r="C34" s="46" t="s">
         <v>357</v>
       </c>
       <c r="D34" s="38" t="s">
-        <v>552</v>
+        <v>549</v>
       </c>
       <c r="E34" s="47" t="s">
         <v>33</v>
@@ -9306,7 +9306,7 @@
         <v>358</v>
       </c>
       <c r="D35" s="38" t="s">
-        <v>551</v>
+        <v>548</v>
       </c>
       <c r="E35" s="47" t="s">
         <v>33</v>
@@ -9323,13 +9323,13 @@
         <v>274</v>
       </c>
       <c r="B36" s="45" t="s">
-        <v>562</v>
+        <v>559</v>
       </c>
       <c r="C36" s="46" t="s">
         <v>359</v>
       </c>
       <c r="D36" s="52" t="s">
-        <v>575</v>
+        <v>572</v>
       </c>
       <c r="E36" s="47" t="s">
         <v>67</v>
@@ -9352,7 +9352,7 @@
         <v>360</v>
       </c>
       <c r="D37" s="52" t="s">
-        <v>576</v>
+        <v>573</v>
       </c>
       <c r="E37" s="47" t="s">
         <v>67</v>
@@ -9369,13 +9369,13 @@
         <v>274</v>
       </c>
       <c r="B38" s="45" t="s">
-        <v>563</v>
+        <v>560</v>
       </c>
       <c r="C38" s="46" t="s">
         <v>361</v>
       </c>
       <c r="D38" s="38" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="E38" s="47" t="s">
         <v>67</v>
@@ -9392,13 +9392,13 @@
         <v>274</v>
       </c>
       <c r="B39" s="45" t="s">
-        <v>564</v>
+        <v>561</v>
       </c>
       <c r="C39" s="46" t="s">
         <v>362</v>
       </c>
       <c r="D39" s="38" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="E39" s="47" t="s">
         <v>67</v>
@@ -9415,13 +9415,13 @@
         <v>274</v>
       </c>
       <c r="B40" s="45" t="s">
-        <v>565</v>
+        <v>562</v>
       </c>
       <c r="C40" s="46" t="s">
         <v>363</v>
       </c>
       <c r="D40" s="38" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="E40" s="47" t="s">
         <v>67</v>
@@ -9438,13 +9438,13 @@
         <v>274</v>
       </c>
       <c r="B41" s="45" t="s">
-        <v>566</v>
+        <v>563</v>
       </c>
       <c r="C41" s="46" t="s">
         <v>364</v>
       </c>
       <c r="D41" s="38" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="E41" s="47" t="s">
         <v>67</v>
@@ -9467,7 +9467,7 @@
         <v>365</v>
       </c>
       <c r="D42" s="38" t="s">
-        <v>538</v>
+        <v>577</v>
       </c>
       <c r="E42" s="47" t="s">
         <v>402</v>
@@ -9480,13 +9480,13 @@
         <v>275</v>
       </c>
       <c r="B43" s="41" t="s">
-        <v>558</v>
+        <v>555</v>
       </c>
       <c r="C43" s="46" t="s">
         <v>366</v>
       </c>
       <c r="D43" s="38" t="s">
-        <v>539</v>
+        <v>537</v>
       </c>
       <c r="E43" s="47" t="s">
         <v>33</v>
@@ -9503,13 +9503,13 @@
         <v>275</v>
       </c>
       <c r="B44" s="41" t="s">
-        <v>559</v>
+        <v>556</v>
       </c>
       <c r="C44" s="46" t="s">
         <v>367</v>
       </c>
       <c r="D44" s="38" t="s">
-        <v>540</v>
+        <v>538</v>
       </c>
       <c r="E44" s="47" t="s">
         <v>33</v>
@@ -9526,13 +9526,13 @@
         <v>275</v>
       </c>
       <c r="B45" s="41" t="s">
-        <v>560</v>
+        <v>557</v>
       </c>
       <c r="C45" s="46" t="s">
         <v>368</v>
       </c>
       <c r="D45" s="38" t="s">
-        <v>541</v>
+        <v>539</v>
       </c>
       <c r="E45" s="47" t="s">
         <v>33</v>
@@ -9549,13 +9549,13 @@
         <v>275</v>
       </c>
       <c r="B46" s="41" t="s">
-        <v>557</v>
+        <v>554</v>
       </c>
       <c r="C46" s="46" t="s">
         <v>369</v>
       </c>
       <c r="D46" s="38" t="s">
-        <v>556</v>
+        <v>553</v>
       </c>
       <c r="E46" s="47" t="s">
         <v>33</v>
@@ -9578,7 +9578,7 @@
         <v>370</v>
       </c>
       <c r="D47" s="38" t="s">
-        <v>542</v>
+        <v>540</v>
       </c>
       <c r="E47" s="47" t="s">
         <v>33</v>
@@ -9595,13 +9595,13 @@
         <v>275</v>
       </c>
       <c r="B48" s="41" t="s">
-        <v>561</v>
+        <v>558</v>
       </c>
       <c r="C48" s="46" t="s">
         <v>371</v>
       </c>
       <c r="D48" s="38" t="s">
-        <v>555</v>
+        <v>552</v>
       </c>
       <c r="E48" s="47" t="s">
         <v>33</v>
@@ -9624,7 +9624,7 @@
         <v>372</v>
       </c>
       <c r="D49" s="38" t="s">
-        <v>554</v>
+        <v>551</v>
       </c>
       <c r="E49" s="47" t="s">
         <v>33</v>
@@ -9641,13 +9641,13 @@
         <v>275</v>
       </c>
       <c r="B50" s="45" t="s">
-        <v>567</v>
+        <v>564</v>
       </c>
       <c r="C50" s="46" t="s">
         <v>373</v>
       </c>
       <c r="D50" s="52" t="s">
-        <v>577</v>
+        <v>574</v>
       </c>
       <c r="E50" s="47" t="s">
         <v>67</v>
@@ -9664,13 +9664,13 @@
         <v>275</v>
       </c>
       <c r="B51" s="45" t="s">
-        <v>562</v>
+        <v>559</v>
       </c>
       <c r="C51" s="46" t="s">
         <v>374</v>
       </c>
       <c r="D51" s="52" t="s">
-        <v>578</v>
+        <v>575</v>
       </c>
       <c r="E51" s="47" t="s">
         <v>67</v>
@@ -9687,13 +9687,13 @@
         <v>275</v>
       </c>
       <c r="B52" s="45" t="s">
-        <v>563</v>
+        <v>560</v>
       </c>
       <c r="C52" s="46" t="s">
         <v>375</v>
       </c>
       <c r="D52" s="38" t="s">
-        <v>543</v>
+        <v>541</v>
       </c>
       <c r="E52" s="47" t="s">
         <v>67</v>
@@ -9710,13 +9710,13 @@
         <v>275</v>
       </c>
       <c r="B53" s="45" t="s">
-        <v>564</v>
+        <v>561</v>
       </c>
       <c r="C53" s="46" t="s">
         <v>376</v>
       </c>
       <c r="D53" s="38" t="s">
-        <v>544</v>
+        <v>542</v>
       </c>
       <c r="E53" s="47" t="s">
         <v>67</v>
@@ -9733,13 +9733,13 @@
         <v>275</v>
       </c>
       <c r="B54" s="45" t="s">
-        <v>565</v>
+        <v>562</v>
       </c>
       <c r="C54" s="46" t="s">
         <v>377</v>
       </c>
       <c r="D54" s="38" t="s">
-        <v>545</v>
+        <v>543</v>
       </c>
       <c r="E54" s="47" t="s">
         <v>67</v>
@@ -9756,13 +9756,13 @@
         <v>275</v>
       </c>
       <c r="B55" s="45" t="s">
-        <v>566</v>
+        <v>563</v>
       </c>
       <c r="C55" s="46" t="s">
         <v>378</v>
       </c>
       <c r="D55" s="38" t="s">
-        <v>545</v>
+        <v>543</v>
       </c>
       <c r="E55" s="47" t="s">
         <v>67</v>
@@ -9785,7 +9785,7 @@
         <v>379</v>
       </c>
       <c r="D56" s="38" t="s">
-        <v>546</v>
+        <v>578</v>
       </c>
       <c r="E56" s="47" t="s">
         <v>402</v>
@@ -10214,21 +10214,21 @@
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="B11:D11"/>
+    <mergeCell ref="B12:D12"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="B14:D14"/>
+    <mergeCell ref="B15:D15"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="B10:D10"/>
     <mergeCell ref="B1:D1"/>
     <mergeCell ref="B2:D2"/>
     <mergeCell ref="B3:D3"/>
     <mergeCell ref="B4:D4"/>
     <mergeCell ref="B5:D5"/>
-    <mergeCell ref="B6:D6"/>
-    <mergeCell ref="B7:D7"/>
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="B9:D9"/>
-    <mergeCell ref="B10:D10"/>
-    <mergeCell ref="B11:D11"/>
-    <mergeCell ref="B12:D12"/>
-    <mergeCell ref="B13:D13"/>
-    <mergeCell ref="B14:D14"/>
-    <mergeCell ref="B15:D15"/>
   </mergeCells>
   <phoneticPr fontId="12" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -10664,22 +10664,22 @@
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="B1:D1"/>
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="B10:D10"/>
     <mergeCell ref="B16:D16"/>
     <mergeCell ref="B11:D11"/>
     <mergeCell ref="B12:D12"/>
     <mergeCell ref="B13:D13"/>
     <mergeCell ref="B14:D14"/>
     <mergeCell ref="B15:D15"/>
-    <mergeCell ref="B6:D6"/>
-    <mergeCell ref="B7:D7"/>
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="B9:D9"/>
-    <mergeCell ref="B10:D10"/>
-    <mergeCell ref="B1:D1"/>
-    <mergeCell ref="B2:D2"/>
-    <mergeCell ref="B3:D3"/>
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="B5:D5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -11313,6 +11313,16 @@
     </row>
   </sheetData>
   <mergeCells count="24">
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="B14:D14"/>
+    <mergeCell ref="B15:D15"/>
+    <mergeCell ref="B1:D1"/>
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="B5:D5"/>
     <mergeCell ref="B22:D22"/>
     <mergeCell ref="B23:D23"/>
     <mergeCell ref="B24:D24"/>
@@ -11327,16 +11337,6 @@
     <mergeCell ref="B19:D19"/>
     <mergeCell ref="B20:D20"/>
     <mergeCell ref="B21:D21"/>
-    <mergeCell ref="B1:D1"/>
-    <mergeCell ref="B2:D2"/>
-    <mergeCell ref="B3:D3"/>
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="B5:D5"/>
-    <mergeCell ref="B6:D6"/>
-    <mergeCell ref="B7:D7"/>
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="B14:D14"/>
-    <mergeCell ref="B15:D15"/>
   </mergeCells>
   <phoneticPr fontId="12" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -11718,11 +11718,6 @@
     </row>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="B2:D2"/>
-    <mergeCell ref="B1:D1"/>
-    <mergeCell ref="B3:D3"/>
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="B5:D5"/>
     <mergeCell ref="B11:D11"/>
     <mergeCell ref="B12:D12"/>
     <mergeCell ref="B13:D13"/>
@@ -11732,6 +11727,11 @@
     <mergeCell ref="B8:D8"/>
     <mergeCell ref="B9:D9"/>
     <mergeCell ref="B10:D10"/>
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="B1:D1"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="B5:D5"/>
   </mergeCells>
   <phoneticPr fontId="12" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -11754,11 +11754,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="58" t="s">
+      <c r="A1" s="59" t="s">
         <v>455</v>
       </c>
-      <c r="B1" s="58"/>
-      <c r="C1" s="58"/>
+      <c r="B1" s="59"/>
+      <c r="C1" s="59"/>
       <c r="D1" s="32" t="s">
         <v>0</v>
       </c>
@@ -11776,11 +11776,11 @@
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A2" s="58" t="s">
+      <c r="A2" s="59" t="s">
         <v>446</v>
       </c>
-      <c r="B2" s="58"/>
-      <c r="C2" s="58"/>
+      <c r="B2" s="59"/>
+      <c r="C2" s="59"/>
       <c r="D2" s="32" t="s">
         <v>1</v>
       </c>
@@ -11798,11 +11798,11 @@
       </c>
     </row>
     <row r="3" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="58" t="s">
+      <c r="A3" s="59" t="s">
         <v>451</v>
       </c>
-      <c r="B3" s="58"/>
-      <c r="C3" s="58"/>
+      <c r="B3" s="59"/>
+      <c r="C3" s="59"/>
       <c r="D3" s="32" t="s">
         <v>3</v>
       </c>
@@ -11820,11 +11820,11 @@
       </c>
     </row>
     <row r="4" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A4" s="58" t="s">
+      <c r="A4" s="59" t="s">
         <v>452</v>
       </c>
-      <c r="B4" s="58"/>
-      <c r="C4" s="58"/>
+      <c r="B4" s="59"/>
+      <c r="C4" s="59"/>
       <c r="D4" s="32" t="s">
         <v>5</v>
       </c>
@@ -11842,11 +11842,11 @@
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" s="58" t="s">
+      <c r="A5" s="59" t="s">
         <v>486</v>
       </c>
-      <c r="B5" s="58"/>
-      <c r="C5" s="58"/>
+      <c r="B5" s="59"/>
+      <c r="C5" s="59"/>
       <c r="D5" s="32" t="s">
         <v>7</v>
       </c>
@@ -11864,11 +11864,11 @@
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A6" s="58" t="s">
+      <c r="A6" s="59" t="s">
         <v>487</v>
       </c>
-      <c r="B6" s="58"/>
-      <c r="C6" s="58"/>
+      <c r="B6" s="59"/>
+      <c r="C6" s="59"/>
       <c r="D6" s="32" t="s">
         <v>9</v>
       </c>
@@ -11886,11 +11886,11 @@
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A7" s="59" t="s">
+      <c r="A7" s="58" t="s">
         <v>488</v>
       </c>
-      <c r="B7" s="59"/>
-      <c r="C7" s="59"/>
+      <c r="B7" s="58"/>
+      <c r="C7" s="58"/>
       <c r="D7" s="32" t="s">
         <v>12</v>
       </c>
@@ -11908,11 +11908,11 @@
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" s="59" t="s">
+      <c r="A8" s="58" t="s">
         <v>489</v>
       </c>
-      <c r="B8" s="59"/>
-      <c r="C8" s="59"/>
+      <c r="B8" s="58"/>
+      <c r="C8" s="58"/>
       <c r="D8" s="32" t="s">
         <v>14</v>
       </c>
@@ -11930,11 +11930,11 @@
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" s="59" t="s">
+      <c r="A9" s="58" t="s">
         <v>490</v>
       </c>
-      <c r="B9" s="59"/>
-      <c r="C9" s="59"/>
+      <c r="B9" s="58"/>
+      <c r="C9" s="58"/>
       <c r="D9" s="32" t="s">
         <v>16</v>
       </c>
@@ -11952,11 +11952,11 @@
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" s="59" t="s">
+      <c r="A10" s="58" t="s">
         <v>491</v>
       </c>
-      <c r="B10" s="59"/>
-      <c r="C10" s="59"/>
+      <c r="B10" s="58"/>
+      <c r="C10" s="58"/>
       <c r="D10" s="32" t="s">
         <v>18</v>
       </c>
@@ -11983,16 +11983,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="A5:C5"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A1:C1"/>
     <mergeCell ref="A9:C9"/>
     <mergeCell ref="A10:C10"/>
     <mergeCell ref="A8:C8"/>
     <mergeCell ref="A7:C7"/>
     <mergeCell ref="A6:C6"/>
-    <mergeCell ref="A5:C5"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="A3:C3"/>
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="A1:C1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -12012,11 +12012,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="58" t="s">
+      <c r="A1" s="59" t="s">
         <v>455</v>
       </c>
-      <c r="B1" s="58"/>
-      <c r="C1" s="58"/>
+      <c r="B1" s="59"/>
+      <c r="C1" s="59"/>
       <c r="D1" s="32" t="s">
         <v>0</v>
       </c>
@@ -12034,11 +12034,11 @@
       </c>
     </row>
     <row r="2" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="58" t="s">
+      <c r="A2" s="59" t="s">
         <v>446</v>
       </c>
-      <c r="B2" s="58"/>
-      <c r="C2" s="58"/>
+      <c r="B2" s="59"/>
+      <c r="C2" s="59"/>
       <c r="D2" s="32" t="s">
         <v>1</v>
       </c>
@@ -12056,11 +12056,11 @@
       </c>
     </row>
     <row r="3" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="58" t="s">
+      <c r="A3" s="59" t="s">
         <v>451</v>
       </c>
-      <c r="B3" s="58"/>
-      <c r="C3" s="58"/>
+      <c r="B3" s="59"/>
+      <c r="C3" s="59"/>
       <c r="D3" s="32" t="s">
         <v>3</v>
       </c>
@@ -12078,11 +12078,11 @@
       </c>
     </row>
     <row r="4" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A4" s="58" t="s">
+      <c r="A4" s="59" t="s">
         <v>452</v>
       </c>
-      <c r="B4" s="58"/>
-      <c r="C4" s="58"/>
+      <c r="B4" s="59"/>
+      <c r="C4" s="59"/>
       <c r="D4" s="32" t="s">
         <v>5</v>
       </c>
@@ -12100,11 +12100,11 @@
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" s="58" t="s">
+      <c r="A5" s="59" t="s">
         <v>486</v>
       </c>
-      <c r="B5" s="58"/>
-      <c r="C5" s="58"/>
+      <c r="B5" s="59"/>
+      <c r="C5" s="59"/>
       <c r="D5" s="32" t="s">
         <v>7</v>
       </c>
@@ -12122,11 +12122,11 @@
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" s="58" t="s">
+      <c r="A6" s="59" t="s">
         <v>487</v>
       </c>
-      <c r="B6" s="58"/>
-      <c r="C6" s="58"/>
+      <c r="B6" s="59"/>
+      <c r="C6" s="59"/>
       <c r="D6" s="32" t="s">
         <v>9</v>
       </c>
@@ -12145,11 +12145,11 @@
       <c r="I6" s="8"/>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" s="59" t="s">
+      <c r="A7" s="58" t="s">
         <v>488</v>
       </c>
-      <c r="B7" s="59"/>
-      <c r="C7" s="59"/>
+      <c r="B7" s="58"/>
+      <c r="C7" s="58"/>
       <c r="D7" s="32" t="s">
         <v>12</v>
       </c>
@@ -12167,11 +12167,11 @@
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" s="59" t="s">
+      <c r="A8" s="58" t="s">
         <v>489</v>
       </c>
-      <c r="B8" s="59"/>
-      <c r="C8" s="59"/>
+      <c r="B8" s="58"/>
+      <c r="C8" s="58"/>
       <c r="D8" s="32" t="s">
         <v>14</v>
       </c>
@@ -12189,11 +12189,11 @@
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9" s="59" t="s">
+      <c r="A9" s="58" t="s">
         <v>490</v>
       </c>
-      <c r="B9" s="59"/>
-      <c r="C9" s="59"/>
+      <c r="B9" s="58"/>
+      <c r="C9" s="58"/>
       <c r="D9" s="32" t="s">
         <v>16</v>
       </c>
@@ -12211,11 +12211,11 @@
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A10" s="59" t="s">
+      <c r="A10" s="58" t="s">
         <v>491</v>
       </c>
-      <c r="B10" s="59"/>
-      <c r="C10" s="59"/>
+      <c r="B10" s="58"/>
+      <c r="C10" s="58"/>
       <c r="D10" s="32" t="s">
         <v>18</v>
       </c>
@@ -12940,6 +12940,13 @@
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="A10:C10"/>
+    <mergeCell ref="A9:C9"/>
+    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="A14:C14"/>
+    <mergeCell ref="A13:C13"/>
+    <mergeCell ref="A12:C12"/>
+    <mergeCell ref="A11:C11"/>
     <mergeCell ref="A3:C3"/>
     <mergeCell ref="A2:C2"/>
     <mergeCell ref="A1:C1"/>
@@ -12948,13 +12955,6 @@
     <mergeCell ref="A6:C6"/>
     <mergeCell ref="A5:C5"/>
     <mergeCell ref="A4:C4"/>
-    <mergeCell ref="A10:C10"/>
-    <mergeCell ref="A9:C9"/>
-    <mergeCell ref="A15:C15"/>
-    <mergeCell ref="A14:C14"/>
-    <mergeCell ref="A13:C13"/>
-    <mergeCell ref="A12:C12"/>
-    <mergeCell ref="A11:C11"/>
   </mergeCells>
   <phoneticPr fontId="12" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
UI Dong Co Khu s, Khu Khi Khoi
</commit_message>
<xml_diff>
--- a/public/TagWarning.xlsx
+++ b/public/TagWarning.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24131"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83EE638B-6596-4206-9343-90256256D219}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C67AE7D-B6FD-47AA-B370-C1AE4A127CEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="10" activeTab="16" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="16" activeTab="17" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LBMT_PLDM#1" sheetId="1" r:id="rId1"/>
@@ -25,18 +25,30 @@
     <sheet name="NH1OngKhoiVaQuatGioTK1" sheetId="15" r:id="rId15"/>
     <sheet name="NH2OngKhoiVaQuatGioTK2" sheetId="16" r:id="rId16"/>
     <sheet name="LMV_VeVien" sheetId="19" r:id="rId17"/>
+    <sheet name="DCKhuKhiKhoi" sheetId="20" r:id="rId18"/>
+    <sheet name="DCKhuS" sheetId="21" r:id="rId19"/>
+    <sheet name="LoQuayVeVien" sheetId="22" r:id="rId20"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2013" uniqueCount="579">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2764" uniqueCount="860">
   <si>
     <t>Tag0</t>
   </si>
@@ -1773,13 +1785,856 @@
   </si>
   <si>
     <t>CT_HF4</t>
+  </si>
+  <si>
+    <t>Quạt dẫn scr1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nhiệt độ cuộn dây Pha A </t>
+  </si>
+  <si>
+    <t>TE1159_AIM</t>
+  </si>
+  <si>
+    <t>Nhiệt độ cuộn dây Pha B</t>
+  </si>
+  <si>
+    <t>TE1161_AIM</t>
+  </si>
+  <si>
+    <t>Nhiệt độ cuộn dây Pha C</t>
+  </si>
+  <si>
+    <t>TE1163_AIM</t>
+  </si>
+  <si>
+    <t>TE1157_AIM</t>
+  </si>
+  <si>
+    <t>TE1158_AIM</t>
+  </si>
+  <si>
+    <t>XE1152X_AIM</t>
+  </si>
+  <si>
+    <t>XE1152Y_AIM</t>
+  </si>
+  <si>
+    <t>XE1153X_AIM</t>
+  </si>
+  <si>
+    <t>XE1153Y_AIM</t>
+  </si>
+  <si>
+    <t>Nhiệt độ vòng bi trước quạt</t>
+  </si>
+  <si>
+    <t>TE1151_AIM</t>
+  </si>
+  <si>
+    <t>Nhiệt độ vòng bi sau quạt</t>
+  </si>
+  <si>
+    <t>TE1153_AIM</t>
+  </si>
+  <si>
+    <t>Nhiệt độ vòng bi giữa quạt</t>
+  </si>
+  <si>
+    <t>TE1155_AIM</t>
+  </si>
+  <si>
+    <t>XE1151X_AIM</t>
+  </si>
+  <si>
+    <t>XE1151Y_AIM</t>
+  </si>
+  <si>
+    <t>Dòng điện SCR1</t>
+  </si>
+  <si>
+    <t>AH108_DL_AIM</t>
+  </si>
+  <si>
+    <t>Quạt dẫn scr2</t>
+  </si>
+  <si>
+    <t>TE2159_AIM</t>
+  </si>
+  <si>
+    <t>TE2161_AIM</t>
+  </si>
+  <si>
+    <t>TE2163_AIM</t>
+  </si>
+  <si>
+    <t>TE2157_AIM</t>
+  </si>
+  <si>
+    <t>TE2158_AIM</t>
+  </si>
+  <si>
+    <t>XE2152X_AIM</t>
+  </si>
+  <si>
+    <t>XE2152Y_AIM</t>
+  </si>
+  <si>
+    <t>XE2153X_AIM</t>
+  </si>
+  <si>
+    <t>XE2153Y_AIM</t>
+  </si>
+  <si>
+    <t>TE2151_AIM</t>
+  </si>
+  <si>
+    <t>TE2153_AIM</t>
+  </si>
+  <si>
+    <t>TE2155_AIM</t>
+  </si>
+  <si>
+    <t>XE2151X_AIM</t>
+  </si>
+  <si>
+    <t>XE2151Y_AIM</t>
+  </si>
+  <si>
+    <t>Dòng điện SCR2</t>
+  </si>
+  <si>
+    <t>AH208_DL_AIM</t>
+  </si>
+  <si>
+    <t>Bơi nc tuần hoàn A</t>
+  </si>
+  <si>
+    <t>Nhiệt độ cuộn dây U</t>
+  </si>
+  <si>
+    <t>TE1505_AIM</t>
+  </si>
+  <si>
+    <t>Nhiệt độ cuộn dây V</t>
+  </si>
+  <si>
+    <t>TE1506_AIM</t>
+  </si>
+  <si>
+    <t>Nhiệt độ cuộn dây W</t>
+  </si>
+  <si>
+    <t>TE1507_AIM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nhiệt độ vào bi dẫn động </t>
+  </si>
+  <si>
+    <t>TE1508_AIM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nhiệt độ vào bi không dẫn động </t>
+  </si>
+  <si>
+    <t>TE1509_AIM</t>
+  </si>
+  <si>
+    <t>Dòng điện bơi nước tuần hoàn A</t>
+  </si>
+  <si>
+    <t>AH107_DL_AIM</t>
+  </si>
+  <si>
+    <t>Bơi nc tuần hoàn B</t>
+  </si>
+  <si>
+    <t>TE1510_AIM</t>
+  </si>
+  <si>
+    <t>TE1511_AIM</t>
+  </si>
+  <si>
+    <t>TE1512_AIM</t>
+  </si>
+  <si>
+    <t>TE1513_AIM</t>
+  </si>
+  <si>
+    <t>TE1514_AIM</t>
+  </si>
+  <si>
+    <t>Dòng điện bơi nước tuần hoàn B</t>
+  </si>
+  <si>
+    <t>AH206_DL_AIM</t>
+  </si>
+  <si>
+    <t>Bơi nc tuần hoàn C</t>
+  </si>
+  <si>
+    <t>TE1515_AIM</t>
+  </si>
+  <si>
+    <t>TE1516_AIM</t>
+  </si>
+  <si>
+    <t>TE1517_AIM</t>
+  </si>
+  <si>
+    <t>TE1518_AIM</t>
+  </si>
+  <si>
+    <t>TE1519_AIM</t>
+  </si>
+  <si>
+    <t>Dòng điện bơi nước tuần hoàn C</t>
+  </si>
+  <si>
+    <t>AH106_DL_AIM</t>
+  </si>
+  <si>
+    <t>Bơi nc tuần hoàn D</t>
+  </si>
+  <si>
+    <t>TE1520_AIM</t>
+  </si>
+  <si>
+    <t>TE1521_AIM</t>
+  </si>
+  <si>
+    <t>TE1522_AIM</t>
+  </si>
+  <si>
+    <t>TE1523_AIM</t>
+  </si>
+  <si>
+    <t>TE1524_AIM</t>
+  </si>
+  <si>
+    <t>Dòng điện bơi nước tuần hoàn D</t>
+  </si>
+  <si>
+    <t>AH207_DL_AIM</t>
+  </si>
+  <si>
+    <t>Độ rung gối trước động cơ trục (X)</t>
+  </si>
+  <si>
+    <t>Độ rung gối sau động cơ trục (X)</t>
+  </si>
+  <si>
+    <t>Độ rung gối trước động cơ  trục (Y)</t>
+  </si>
+  <si>
+    <t>Độ rung gối sau động cơ trục (Y)</t>
+  </si>
+  <si>
+    <t>Độ rung gối quạt trục (X)</t>
+  </si>
+  <si>
+    <t>Độ rung gối quạt trục (Y)</t>
+  </si>
+  <si>
+    <t>mm/S</t>
+  </si>
+  <si>
+    <t>Quạt tăng áp 1A</t>
+  </si>
+  <si>
+    <t>Os_1A_ZYFJ_DJ_U_TT</t>
+  </si>
+  <si>
+    <t>Os_1A_ZYFJ_DJ_V_TT</t>
+  </si>
+  <si>
+    <t>Os_1A_ZYFJ_DJ_W_TT</t>
+  </si>
+  <si>
+    <t>Os_1A_ZYFJ_DJ_QZC_TT</t>
+  </si>
+  <si>
+    <t>Os_1A_ZYFJ_DJ_HZC_TT</t>
+  </si>
+  <si>
+    <t>Nhiệt độ gối quạt tăng áp #1</t>
+  </si>
+  <si>
+    <t>Os_1A_ZYFJ_FJZC_TT_1</t>
+  </si>
+  <si>
+    <t>Nhiệt độ gối quạt tăng áp #2</t>
+  </si>
+  <si>
+    <t>Os_1A_ZYFJ_FJZC_TT_2</t>
+  </si>
+  <si>
+    <t>Nhiệt độ gối quạt tăng áp #3</t>
+  </si>
+  <si>
+    <t>Os_1A_ZYFJ_FJZC_TT_3</t>
+  </si>
+  <si>
+    <t>Os_1A_ZYFJ_FJ_X_VIB</t>
+  </si>
+  <si>
+    <t>Os_1A_ZYFJ_FJ_Y_VIB</t>
+  </si>
+  <si>
+    <t>Os_1A_ZYFJ_QZC_VIB</t>
+  </si>
+  <si>
+    <t>Os_1A_ZYFJ_HZC_VIB</t>
+  </si>
+  <si>
+    <t>Os_1_8AH_IL2</t>
+  </si>
+  <si>
+    <t>Quạt tăng áp 1B</t>
+  </si>
+  <si>
+    <t>Os_1B_ZYFJ_DJ_U_TT</t>
+  </si>
+  <si>
+    <t>Os_1B_ZYFJ_DJ_V_TT</t>
+  </si>
+  <si>
+    <t>Os_1B_ZYFJ_DJ_W_TT</t>
+  </si>
+  <si>
+    <t>Os_1B_ZYFJ_DJ_QZC_TT</t>
+  </si>
+  <si>
+    <t>Os_1B_ZYFJ_DJ_HZC_TT</t>
+  </si>
+  <si>
+    <t>Os_1B_ZYFJ_FJZC_TT_1</t>
+  </si>
+  <si>
+    <t>Os_1B_ZYFJ_FJZC_TT_2</t>
+  </si>
+  <si>
+    <t>Os_1B_ZYFJ_FJZC_TT_3</t>
+  </si>
+  <si>
+    <t>Os_1B_ZYFJ_FJ_X_VIB</t>
+  </si>
+  <si>
+    <t>Os_1B_ZYFJ_FJ_Y_VIB</t>
+  </si>
+  <si>
+    <t>Os_1B_ZYFJ_QZC_VIB</t>
+  </si>
+  <si>
+    <t>Os_1B_ZYFJ_HZC_VIB</t>
+  </si>
+  <si>
+    <t>Os_1_9AH_IL2</t>
+  </si>
+  <si>
+    <t>Quạt tăng áp 2A</t>
+  </si>
+  <si>
+    <t>Os_2A_ZYFJ_DJ_U_TT</t>
+  </si>
+  <si>
+    <t>Os_2A_ZYFJ_DJ_V_TT</t>
+  </si>
+  <si>
+    <t>Os_2A_ZYFJ_DJ_W_TT</t>
+  </si>
+  <si>
+    <t>Os_2A_ZYFJ_DJ_QZC_TT</t>
+  </si>
+  <si>
+    <t>Os_2A_ZYFJ_DJ_HZC_TT</t>
+  </si>
+  <si>
+    <t>Os_2A_ZYFJ_FJZC_TT_1</t>
+  </si>
+  <si>
+    <t>Os_2A_ZYFJ_FJZC_TT_2</t>
+  </si>
+  <si>
+    <t>Os_2A_ZYFJ_FJZC_TT_3</t>
+  </si>
+  <si>
+    <t>Os_2A_ZYFJ_FJ_X_VIB</t>
+  </si>
+  <si>
+    <t>Os_2A_ZYFJ_FJ_Y_VIB</t>
+  </si>
+  <si>
+    <t>Os_2A_ZYFJ_QZC_VIB</t>
+  </si>
+  <si>
+    <t>Os_2A_ZYFJ_HZC_VIB</t>
+  </si>
+  <si>
+    <t>Os_2_8AH_IL2</t>
+  </si>
+  <si>
+    <t>Quạt tăng áp 2B</t>
+  </si>
+  <si>
+    <t>Os_2B_ZYFJ_DJ_U_TT</t>
+  </si>
+  <si>
+    <t>Os_2B_ZYFJ_DJ_V_TT</t>
+  </si>
+  <si>
+    <t>Os_2B_ZYFJ_DJ_W_TT</t>
+  </si>
+  <si>
+    <t>Os_2B_ZYFJ_DJ_QZC_TT</t>
+  </si>
+  <si>
+    <t>Os_2B_ZYFJ_DJ_HZC_TT</t>
+  </si>
+  <si>
+    <t>Os_2B_ZYFJ_FJZC_TT_1</t>
+  </si>
+  <si>
+    <t>Os_2B_ZYFJ_FJZC_TT_2</t>
+  </si>
+  <si>
+    <t>Os_2B_ZYFJ_FJZC_TT_3</t>
+  </si>
+  <si>
+    <t>Os_2B_ZYFJ_FJ_X_VIB</t>
+  </si>
+  <si>
+    <t>Os_2B_ZYFJ_FJ_Y_VIB</t>
+  </si>
+  <si>
+    <t>Os_2B_ZYFJ_QZC_VIB</t>
+  </si>
+  <si>
+    <t>Os_2B_ZYFJ_HZC_VIB</t>
+  </si>
+  <si>
+    <t>Os_2_9AH_IL2</t>
+  </si>
+  <si>
+    <t>Os_1A_JYXHB_DJ_U_TT</t>
+  </si>
+  <si>
+    <t>Os_1A_JYXHB_DJ_V_TT</t>
+  </si>
+  <si>
+    <t>Os_1A_JYXHB_DJ_W_TT</t>
+  </si>
+  <si>
+    <t>Os_1A_JYXHB_DJ_QZC_TT</t>
+  </si>
+  <si>
+    <t>Os_1A_JYXHB_DJ_HZC_TT</t>
+  </si>
+  <si>
+    <t>Os_1A_JYXHB_ZC_TT_1</t>
+  </si>
+  <si>
+    <t>Os_1A_JYXHB_ZC_TT_2</t>
+  </si>
+  <si>
+    <t>Os_1_4AH_IL2</t>
+  </si>
+  <si>
+    <t>Os_1B_JYXHB_DJ_U_TT</t>
+  </si>
+  <si>
+    <t>Os_1B_JYXHB_DJ_V_TT</t>
+  </si>
+  <si>
+    <t>Os_1B_JYXHB_DJ_W_TT</t>
+  </si>
+  <si>
+    <t>Os_1B_JYXHB_DJ_QZC_TT</t>
+  </si>
+  <si>
+    <t>Os_1B_JYXHB_DJ_HZC_TT</t>
+  </si>
+  <si>
+    <t>Os_1B_JYXHB_ZC_TT_1</t>
+  </si>
+  <si>
+    <t>Os_1B_JYXHB_ZC_TT_2</t>
+  </si>
+  <si>
+    <t>Os_1_5AH_IL2</t>
+  </si>
+  <si>
+    <t>Os_1C_JYXHB_DJ_U_TT</t>
+  </si>
+  <si>
+    <t>Os_1C_JYXHB_DJ_V_TT</t>
+  </si>
+  <si>
+    <t>Os_1C_JYXHB_DJ_W_TT</t>
+  </si>
+  <si>
+    <t>Os_1C_JYXHB_DJ_QZC_TT</t>
+  </si>
+  <si>
+    <t>Os_1C_JYXHB_DJ_HZC_TT</t>
+  </si>
+  <si>
+    <t>Os_1C_JYXHB_ZC_TT_1</t>
+  </si>
+  <si>
+    <t>Os_1C_JYXHB_ZC_TT_2</t>
+  </si>
+  <si>
+    <t>Os_1_6AH_IL2</t>
+  </si>
+  <si>
+    <t>Os_1D_JYXHB_DJ_U_TT</t>
+  </si>
+  <si>
+    <t>Os_1D_JYXHB_DJ_V_TT</t>
+  </si>
+  <si>
+    <t>Os_1D_JYXHB_DJ_W_TT</t>
+  </si>
+  <si>
+    <t>Os_1D_JYXHB_DJ_QZC_TT</t>
+  </si>
+  <si>
+    <t>Os_1D_JYXHB_DJ_HZC_TT</t>
+  </si>
+  <si>
+    <t>Os_1D_JYXHB_ZC_TT_1</t>
+  </si>
+  <si>
+    <t>Os_1D_JYXHB_ZC_TT_2</t>
+  </si>
+  <si>
+    <t>Os_1_7AH_IL2</t>
+  </si>
+  <si>
+    <t>Os_2A_JYXHB_DJ_U_TT</t>
+  </si>
+  <si>
+    <t>Os_2A_JYXHB_DJ_V_TT</t>
+  </si>
+  <si>
+    <t>Os_2A_JYXHB_DJ_W_TT</t>
+  </si>
+  <si>
+    <t>Os_2A_JYXHB_DJ_QZC_TT</t>
+  </si>
+  <si>
+    <t>Os_2A_JYXHB_DJ_HZC_TT</t>
+  </si>
+  <si>
+    <t>Os_2A_JYXHB_ZC_TT_1</t>
+  </si>
+  <si>
+    <t>Os_2A_JYXHB_ZC_TT_2</t>
+  </si>
+  <si>
+    <t>Os_2_4AH_IL2</t>
+  </si>
+  <si>
+    <t>Os_2B_JYXHB_DJ_U_TT</t>
+  </si>
+  <si>
+    <t>Os_2B_JYXHB_DJ_V_TT</t>
+  </si>
+  <si>
+    <t>Os_2B_JYXHB_DJ_W_TT</t>
+  </si>
+  <si>
+    <t>Os_2B_JYXHB_DJ_QZC_TT</t>
+  </si>
+  <si>
+    <t>Os_2B_JYXHB_DJ_HZC_TT</t>
+  </si>
+  <si>
+    <t>Os_2B_JYXHB_ZC_TT_1</t>
+  </si>
+  <si>
+    <t>Os_2B_JYXHB_ZC_TT_2</t>
+  </si>
+  <si>
+    <t>Os_2_5AH_IL2</t>
+  </si>
+  <si>
+    <t>Os_2C_JYXHB_DJ_U_TT</t>
+  </si>
+  <si>
+    <t>Os_2C_JYXHB_DJ_V_TT</t>
+  </si>
+  <si>
+    <t>Os_2C_JYXHB_DJ_W_TT</t>
+  </si>
+  <si>
+    <t>Os_2C_JYXHB_DJ_QZC_TT</t>
+  </si>
+  <si>
+    <t>Os_2C_JYXHB_DJ_HZC_TT</t>
+  </si>
+  <si>
+    <t>Os_2C_JYXHB_ZC_TT_1</t>
+  </si>
+  <si>
+    <t>Os_2C_JYXHB_ZC_TT_2</t>
+  </si>
+  <si>
+    <t>Os_2_6AH_IL2</t>
+  </si>
+  <si>
+    <t>Os_2D_JYXHB_DJ_U_TT</t>
+  </si>
+  <si>
+    <t>Os_2D_JYXHB_DJ_V_TT</t>
+  </si>
+  <si>
+    <t>Os_2D_JYXHB_DJ_W_TT</t>
+  </si>
+  <si>
+    <t>Os_2D_JYXHB_DJ_QZC_TT</t>
+  </si>
+  <si>
+    <t>Os_2D_JYXHB_DJ_HZC_TT</t>
+  </si>
+  <si>
+    <t>Os_2D_JYXHB_ZC_TT_1</t>
+  </si>
+  <si>
+    <t>Os_2D_JYXHB_ZC_TT_2</t>
+  </si>
+  <si>
+    <t>Os_2_7AH_IL2</t>
+  </si>
+  <si>
+    <t>Bơm vữa tuần hoàn 1A</t>
+  </si>
+  <si>
+    <t>Bơm vữa tuần hoàn 1B</t>
+  </si>
+  <si>
+    <t>Bơm vữa tuần hoàn 1C</t>
+  </si>
+  <si>
+    <t>Bơm vữa tuần hoàn 1D</t>
+  </si>
+  <si>
+    <t>Bơm vữa tuần hoàn 2A</t>
+  </si>
+  <si>
+    <t>Bơm vữa tuần hoàn 2B</t>
+  </si>
+  <si>
+    <t>Bơm vữa tuần hoàn 2C</t>
+  </si>
+  <si>
+    <t>Bơm vữa tuần hoàn 2D</t>
+  </si>
+  <si>
+    <t>Tag78</t>
+  </si>
+  <si>
+    <t>Tag79</t>
+  </si>
+  <si>
+    <t>Tag80</t>
+  </si>
+  <si>
+    <t>Tag81</t>
+  </si>
+  <si>
+    <t>Tag82</t>
+  </si>
+  <si>
+    <t>Tag83</t>
+  </si>
+  <si>
+    <t>Tag84</t>
+  </si>
+  <si>
+    <t>Tag85</t>
+  </si>
+  <si>
+    <t>Tag86</t>
+  </si>
+  <si>
+    <t>Tag87</t>
+  </si>
+  <si>
+    <t>Tag88</t>
+  </si>
+  <si>
+    <t>Tag89</t>
+  </si>
+  <si>
+    <t>Tag90</t>
+  </si>
+  <si>
+    <t>Tag91</t>
+  </si>
+  <si>
+    <t>Tag92</t>
+  </si>
+  <si>
+    <t>Tag93</t>
+  </si>
+  <si>
+    <t>Tag94</t>
+  </si>
+  <si>
+    <t>Tag95</t>
+  </si>
+  <si>
+    <t>Tag96</t>
+  </si>
+  <si>
+    <t>Tag97</t>
+  </si>
+  <si>
+    <t>Tag98</t>
+  </si>
+  <si>
+    <t>Tag99</t>
+  </si>
+  <si>
+    <t>Tag100</t>
+  </si>
+  <si>
+    <t>Tag101</t>
+  </si>
+  <si>
+    <t>Tag102</t>
+  </si>
+  <si>
+    <t>Tag103</t>
+  </si>
+  <si>
+    <t>Tag104</t>
+  </si>
+  <si>
+    <t>Tag105</t>
+  </si>
+  <si>
+    <t>Tag106</t>
+  </si>
+  <si>
+    <t>Tag107</t>
+  </si>
+  <si>
+    <t>Tag108</t>
+  </si>
+  <si>
+    <t>Tag109</t>
+  </si>
+  <si>
+    <t>Tag110</t>
+  </si>
+  <si>
+    <t>Tag111</t>
+  </si>
+  <si>
+    <t>Tag112</t>
+  </si>
+  <si>
+    <t>Tag113</t>
+  </si>
+  <si>
+    <t>Tag114</t>
+  </si>
+  <si>
+    <t>Tag115</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nhiệt độ Đầu lò </t>
+  </si>
+  <si>
+    <t>TI704M</t>
+  </si>
+  <si>
+    <t>Nhiệt độ  Vùng nung</t>
+  </si>
+  <si>
+    <t>TI703M</t>
+  </si>
+  <si>
+    <t>Nhiệt độ  Đuôi lò</t>
+  </si>
+  <si>
+    <t>TI705M</t>
+  </si>
+  <si>
+    <t>YY_SETPOINT1</t>
+  </si>
+  <si>
+    <t>SI801aM</t>
+  </si>
+  <si>
+    <t>TI701aM</t>
+  </si>
+  <si>
+    <t>TI701bM</t>
+  </si>
+  <si>
+    <t>TI701cM</t>
+  </si>
+  <si>
+    <t>TI701dM</t>
+  </si>
+  <si>
+    <t>TI701eM</t>
+  </si>
+  <si>
+    <t>TI701fM</t>
+  </si>
+  <si>
+    <t>TI701gM</t>
+  </si>
+  <si>
+    <t>TI701hM</t>
+  </si>
+  <si>
+    <t>Lò Quay</t>
+  </si>
+  <si>
+    <t>%</t>
+  </si>
+  <si>
+    <t>Tốc độ</t>
+  </si>
+  <si>
+    <t>vòng/phút</t>
+  </si>
+  <si>
+    <t>Nhiệt độ vỏ lò điểm nhiệt 1</t>
+  </si>
+  <si>
+    <t>Nhiệt độ vỏ lò điểm nhiệt 2</t>
+  </si>
+  <si>
+    <t>Nhiệt độ vỏ lò điểm nhiệt 3</t>
+  </si>
+  <si>
+    <t>Nhiệt độ vỏ lò điểm nhiệt 4</t>
+  </si>
+  <si>
+    <t>Nhiệt độ vỏ lò điểm nhiệt 5</t>
+  </si>
+  <si>
+    <t>Nhiệt độ vỏ lò điểm nhiệt 6</t>
+  </si>
+  <si>
+    <t>Nhiệt độ vỏ lò điểm nhiệt 7</t>
+  </si>
+  <si>
+    <t>Nhiệt độ vỏ lò điểm nhiệt 8</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="17" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1890,6 +2745,18 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="13"/>
+      <color rgb="FFFF0000"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="13"/>
+      <color rgb="FF1F2937"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -2143,7 +3010,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="77">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2270,10 +3137,10 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2289,6 +3156,36 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2984,12 +3881,6 @@
     </row>
   </sheetData>
   <mergeCells count="16">
-    <mergeCell ref="B1:D1"/>
-    <mergeCell ref="B5:D5"/>
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="B7:D7"/>
-    <mergeCell ref="B6:D6"/>
-    <mergeCell ref="B4:D4"/>
     <mergeCell ref="B16:D16"/>
     <mergeCell ref="B15:D15"/>
     <mergeCell ref="B14:D14"/>
@@ -3000,6 +3891,12 @@
     <mergeCell ref="B11:D11"/>
     <mergeCell ref="B10:D10"/>
     <mergeCell ref="B9:D9"/>
+    <mergeCell ref="B1:D1"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="B4:D4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="261" orientation="landscape" horizontalDpi="180" verticalDpi="180" r:id="rId1"/>
@@ -3360,13 +4257,6 @@
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="A10:C10"/>
-    <mergeCell ref="A9:C9"/>
-    <mergeCell ref="A15:C15"/>
-    <mergeCell ref="A14:C14"/>
-    <mergeCell ref="A13:C13"/>
-    <mergeCell ref="A12:C12"/>
-    <mergeCell ref="A11:C11"/>
     <mergeCell ref="A3:C3"/>
     <mergeCell ref="A2:C2"/>
     <mergeCell ref="A1:C1"/>
@@ -3375,6 +4265,13 @@
     <mergeCell ref="A6:C6"/>
     <mergeCell ref="A5:C5"/>
     <mergeCell ref="A4:C4"/>
+    <mergeCell ref="A10:C10"/>
+    <mergeCell ref="A9:C9"/>
+    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="A14:C14"/>
+    <mergeCell ref="A13:C13"/>
+    <mergeCell ref="A12:C12"/>
+    <mergeCell ref="A11:C11"/>
   </mergeCells>
   <phoneticPr fontId="12" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3765,13 +4662,6 @@
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="A6:C6"/>
-    <mergeCell ref="A7:C7"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="A3:C3"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="A5:C5"/>
     <mergeCell ref="A13:C13"/>
     <mergeCell ref="A14:C14"/>
     <mergeCell ref="A15:C15"/>
@@ -3780,6 +4670,13 @@
     <mergeCell ref="A10:C10"/>
     <mergeCell ref="A11:C11"/>
     <mergeCell ref="A12:C12"/>
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="A7:C7"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="A5:C5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4140,13 +5037,6 @@
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="A6:C6"/>
-    <mergeCell ref="A7:C7"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="A3:C3"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="A5:C5"/>
     <mergeCell ref="A13:C13"/>
     <mergeCell ref="A14:C14"/>
     <mergeCell ref="A15:C15"/>
@@ -4155,6 +5045,13 @@
     <mergeCell ref="A10:C10"/>
     <mergeCell ref="A11:C11"/>
     <mergeCell ref="A12:C12"/>
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="A7:C7"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="A5:C5"/>
   </mergeCells>
   <phoneticPr fontId="12" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -9813,6 +10710,2793 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F8B02CF-8B60-4C10-A1A3-04421F3B73B0}">
+  <dimension ref="A1:G59"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="20" style="39" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="36.85546875" style="39" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.85546875" style="39" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="5.85546875" style="65" bestFit="1" customWidth="1"/>
+    <col min="6" max="16384" width="9.140625" style="39"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A1" s="66" t="s">
+        <v>579</v>
+      </c>
+      <c r="B1" s="38" t="s">
+        <v>580</v>
+      </c>
+      <c r="C1" s="67" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="38" t="s">
+        <v>581</v>
+      </c>
+      <c r="E1" s="68" t="s">
+        <v>33</v>
+      </c>
+      <c r="F1" s="43"/>
+      <c r="G1" s="43"/>
+    </row>
+    <row r="2" spans="1:7" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A2" s="66"/>
+      <c r="B2" s="38" t="s">
+        <v>582</v>
+      </c>
+      <c r="C2" s="67" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="38" t="s">
+        <v>583</v>
+      </c>
+      <c r="E2" s="68" t="s">
+        <v>33</v>
+      </c>
+      <c r="F2" s="43"/>
+      <c r="G2" s="43"/>
+    </row>
+    <row r="3" spans="1:7" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A3" s="66"/>
+      <c r="B3" s="38" t="s">
+        <v>584</v>
+      </c>
+      <c r="C3" s="67" t="s">
+        <v>3</v>
+      </c>
+      <c r="D3" s="38" t="s">
+        <v>585</v>
+      </c>
+      <c r="E3" s="68" t="s">
+        <v>33</v>
+      </c>
+      <c r="F3" s="43"/>
+      <c r="G3" s="43"/>
+    </row>
+    <row r="4" spans="1:7" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A4" s="66"/>
+      <c r="B4" s="38" t="s">
+        <v>215</v>
+      </c>
+      <c r="C4" s="67" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4" s="38" t="s">
+        <v>586</v>
+      </c>
+      <c r="E4" s="68" t="s">
+        <v>33</v>
+      </c>
+      <c r="F4" s="43"/>
+      <c r="G4" s="43"/>
+    </row>
+    <row r="5" spans="1:7" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A5" s="66"/>
+      <c r="B5" s="38" t="s">
+        <v>216</v>
+      </c>
+      <c r="C5" s="67" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="38" t="s">
+        <v>587</v>
+      </c>
+      <c r="E5" s="68" t="s">
+        <v>33</v>
+      </c>
+      <c r="F5" s="43"/>
+      <c r="G5" s="43"/>
+    </row>
+    <row r="6" spans="1:7" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A6" s="66"/>
+      <c r="B6" s="38" t="s">
+        <v>656</v>
+      </c>
+      <c r="C6" s="67" t="s">
+        <v>9</v>
+      </c>
+      <c r="D6" s="38" t="s">
+        <v>588</v>
+      </c>
+      <c r="E6" s="68" t="s">
+        <v>662</v>
+      </c>
+      <c r="F6" s="43"/>
+      <c r="G6" s="43"/>
+    </row>
+    <row r="7" spans="1:7" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A7" s="66"/>
+      <c r="B7" s="38" t="s">
+        <v>658</v>
+      </c>
+      <c r="C7" s="67" t="s">
+        <v>12</v>
+      </c>
+      <c r="D7" s="38" t="s">
+        <v>589</v>
+      </c>
+      <c r="E7" s="68" t="s">
+        <v>662</v>
+      </c>
+      <c r="F7" s="43"/>
+      <c r="G7" s="43"/>
+    </row>
+    <row r="8" spans="1:7" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A8" s="66"/>
+      <c r="B8" s="38" t="s">
+        <v>657</v>
+      </c>
+      <c r="C8" s="67" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" s="38" t="s">
+        <v>590</v>
+      </c>
+      <c r="E8" s="68" t="s">
+        <v>662</v>
+      </c>
+      <c r="F8" s="43"/>
+      <c r="G8" s="43"/>
+    </row>
+    <row r="9" spans="1:7" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A9" s="66"/>
+      <c r="B9" s="38" t="s">
+        <v>659</v>
+      </c>
+      <c r="C9" s="67" t="s">
+        <v>16</v>
+      </c>
+      <c r="D9" s="38" t="s">
+        <v>591</v>
+      </c>
+      <c r="E9" s="68" t="s">
+        <v>662</v>
+      </c>
+      <c r="F9" s="43"/>
+      <c r="G9" s="43"/>
+    </row>
+    <row r="10" spans="1:7" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A10" s="66"/>
+      <c r="B10" s="38" t="s">
+        <v>592</v>
+      </c>
+      <c r="C10" s="67" t="s">
+        <v>18</v>
+      </c>
+      <c r="D10" s="38" t="s">
+        <v>593</v>
+      </c>
+      <c r="E10" s="68" t="s">
+        <v>33</v>
+      </c>
+      <c r="F10" s="43"/>
+      <c r="G10" s="43"/>
+    </row>
+    <row r="11" spans="1:7" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A11" s="66"/>
+      <c r="B11" s="38" t="s">
+        <v>594</v>
+      </c>
+      <c r="C11" s="67" t="s">
+        <v>19</v>
+      </c>
+      <c r="D11" s="38" t="s">
+        <v>595</v>
+      </c>
+      <c r="E11" s="68" t="s">
+        <v>33</v>
+      </c>
+      <c r="F11" s="43"/>
+      <c r="G11" s="43"/>
+    </row>
+    <row r="12" spans="1:7" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A12" s="66"/>
+      <c r="B12" s="38" t="s">
+        <v>596</v>
+      </c>
+      <c r="C12" s="67" t="s">
+        <v>20</v>
+      </c>
+      <c r="D12" s="38" t="s">
+        <v>597</v>
+      </c>
+      <c r="E12" s="68" t="s">
+        <v>33</v>
+      </c>
+      <c r="F12" s="43"/>
+      <c r="G12" s="43"/>
+    </row>
+    <row r="13" spans="1:7" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A13" s="66"/>
+      <c r="B13" s="38" t="s">
+        <v>660</v>
+      </c>
+      <c r="C13" s="67" t="s">
+        <v>21</v>
+      </c>
+      <c r="D13" s="38" t="s">
+        <v>598</v>
+      </c>
+      <c r="E13" s="68" t="s">
+        <v>662</v>
+      </c>
+      <c r="F13" s="43"/>
+      <c r="G13" s="43"/>
+    </row>
+    <row r="14" spans="1:7" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A14" s="66"/>
+      <c r="B14" s="38" t="s">
+        <v>661</v>
+      </c>
+      <c r="C14" s="67" t="s">
+        <v>22</v>
+      </c>
+      <c r="D14" s="38" t="s">
+        <v>599</v>
+      </c>
+      <c r="E14" s="68" t="s">
+        <v>662</v>
+      </c>
+      <c r="F14" s="43"/>
+      <c r="G14" s="43"/>
+    </row>
+    <row r="15" spans="1:7" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A15" s="66"/>
+      <c r="B15" s="69" t="s">
+        <v>600</v>
+      </c>
+      <c r="C15" s="67" t="s">
+        <v>23</v>
+      </c>
+      <c r="D15" s="69" t="s">
+        <v>601</v>
+      </c>
+      <c r="E15" s="70" t="s">
+        <v>402</v>
+      </c>
+      <c r="F15" s="43"/>
+      <c r="G15" s="43"/>
+    </row>
+    <row r="16" spans="1:7" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A16" s="66" t="s">
+        <v>602</v>
+      </c>
+      <c r="B16" s="38" t="s">
+        <v>580</v>
+      </c>
+      <c r="C16" s="67" t="s">
+        <v>24</v>
+      </c>
+      <c r="D16" s="38" t="s">
+        <v>603</v>
+      </c>
+      <c r="E16" s="68" t="s">
+        <v>33</v>
+      </c>
+      <c r="F16" s="43"/>
+      <c r="G16" s="43"/>
+    </row>
+    <row r="17" spans="1:7" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A17" s="66"/>
+      <c r="B17" s="38" t="s">
+        <v>582</v>
+      </c>
+      <c r="C17" s="67" t="s">
+        <v>112</v>
+      </c>
+      <c r="D17" s="38" t="s">
+        <v>604</v>
+      </c>
+      <c r="E17" s="68" t="s">
+        <v>33</v>
+      </c>
+      <c r="F17" s="43"/>
+      <c r="G17" s="43"/>
+    </row>
+    <row r="18" spans="1:7" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A18" s="66"/>
+      <c r="B18" s="38" t="s">
+        <v>584</v>
+      </c>
+      <c r="C18" s="67" t="s">
+        <v>113</v>
+      </c>
+      <c r="D18" s="38" t="s">
+        <v>605</v>
+      </c>
+      <c r="E18" s="68" t="s">
+        <v>33</v>
+      </c>
+      <c r="F18" s="43"/>
+      <c r="G18" s="43"/>
+    </row>
+    <row r="19" spans="1:7" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A19" s="66"/>
+      <c r="B19" s="38" t="s">
+        <v>215</v>
+      </c>
+      <c r="C19" s="67" t="s">
+        <v>114</v>
+      </c>
+      <c r="D19" s="38" t="s">
+        <v>606</v>
+      </c>
+      <c r="E19" s="68" t="s">
+        <v>33</v>
+      </c>
+      <c r="F19" s="43"/>
+      <c r="G19" s="43"/>
+    </row>
+    <row r="20" spans="1:7" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A20" s="66"/>
+      <c r="B20" s="38" t="s">
+        <v>216</v>
+      </c>
+      <c r="C20" s="67" t="s">
+        <v>115</v>
+      </c>
+      <c r="D20" s="38" t="s">
+        <v>607</v>
+      </c>
+      <c r="E20" s="68" t="s">
+        <v>33</v>
+      </c>
+      <c r="F20" s="43"/>
+      <c r="G20" s="43"/>
+    </row>
+    <row r="21" spans="1:7" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A21" s="66"/>
+      <c r="B21" s="38" t="s">
+        <v>656</v>
+      </c>
+      <c r="C21" s="67" t="s">
+        <v>117</v>
+      </c>
+      <c r="D21" s="38" t="s">
+        <v>608</v>
+      </c>
+      <c r="E21" s="68" t="s">
+        <v>662</v>
+      </c>
+      <c r="F21" s="43"/>
+      <c r="G21" s="43"/>
+    </row>
+    <row r="22" spans="1:7" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A22" s="66"/>
+      <c r="B22" s="38" t="s">
+        <v>658</v>
+      </c>
+      <c r="C22" s="67" t="s">
+        <v>119</v>
+      </c>
+      <c r="D22" s="38" t="s">
+        <v>609</v>
+      </c>
+      <c r="E22" s="68" t="s">
+        <v>662</v>
+      </c>
+      <c r="F22" s="43"/>
+      <c r="G22" s="43"/>
+    </row>
+    <row r="23" spans="1:7" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A23" s="66"/>
+      <c r="B23" s="38" t="s">
+        <v>657</v>
+      </c>
+      <c r="C23" s="67" t="s">
+        <v>121</v>
+      </c>
+      <c r="D23" s="38" t="s">
+        <v>610</v>
+      </c>
+      <c r="E23" s="68" t="s">
+        <v>662</v>
+      </c>
+      <c r="F23" s="43"/>
+      <c r="G23" s="43"/>
+    </row>
+    <row r="24" spans="1:7" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A24" s="66"/>
+      <c r="B24" s="38" t="s">
+        <v>659</v>
+      </c>
+      <c r="C24" s="67" t="s">
+        <v>123</v>
+      </c>
+      <c r="D24" s="38" t="s">
+        <v>611</v>
+      </c>
+      <c r="E24" s="68" t="s">
+        <v>662</v>
+      </c>
+      <c r="F24" s="43"/>
+      <c r="G24" s="43"/>
+    </row>
+    <row r="25" spans="1:7" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A25" s="66"/>
+      <c r="B25" s="38" t="s">
+        <v>592</v>
+      </c>
+      <c r="C25" s="67" t="s">
+        <v>348</v>
+      </c>
+      <c r="D25" s="38" t="s">
+        <v>612</v>
+      </c>
+      <c r="E25" s="68" t="s">
+        <v>33</v>
+      </c>
+      <c r="F25" s="43"/>
+      <c r="G25" s="43"/>
+    </row>
+    <row r="26" spans="1:7" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A26" s="66"/>
+      <c r="B26" s="38" t="s">
+        <v>594</v>
+      </c>
+      <c r="C26" s="67" t="s">
+        <v>349</v>
+      </c>
+      <c r="D26" s="38" t="s">
+        <v>613</v>
+      </c>
+      <c r="E26" s="68" t="s">
+        <v>33</v>
+      </c>
+      <c r="F26" s="43"/>
+      <c r="G26" s="43"/>
+    </row>
+    <row r="27" spans="1:7" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A27" s="66"/>
+      <c r="B27" s="38" t="s">
+        <v>596</v>
+      </c>
+      <c r="C27" s="67" t="s">
+        <v>350</v>
+      </c>
+      <c r="D27" s="38" t="s">
+        <v>614</v>
+      </c>
+      <c r="E27" s="68" t="s">
+        <v>33</v>
+      </c>
+      <c r="F27" s="43"/>
+      <c r="G27" s="43"/>
+    </row>
+    <row r="28" spans="1:7" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A28" s="66"/>
+      <c r="B28" s="38" t="s">
+        <v>660</v>
+      </c>
+      <c r="C28" s="67" t="s">
+        <v>351</v>
+      </c>
+      <c r="D28" s="38" t="s">
+        <v>615</v>
+      </c>
+      <c r="E28" s="68" t="s">
+        <v>662</v>
+      </c>
+      <c r="F28" s="43"/>
+      <c r="G28" s="43"/>
+    </row>
+    <row r="29" spans="1:7" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A29" s="66"/>
+      <c r="B29" s="38" t="s">
+        <v>661</v>
+      </c>
+      <c r="C29" s="67" t="s">
+        <v>352</v>
+      </c>
+      <c r="D29" s="38" t="s">
+        <v>616</v>
+      </c>
+      <c r="E29" s="68" t="s">
+        <v>662</v>
+      </c>
+      <c r="F29" s="43"/>
+      <c r="G29" s="43"/>
+    </row>
+    <row r="30" spans="1:7" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A30" s="66"/>
+      <c r="B30" s="69" t="s">
+        <v>617</v>
+      </c>
+      <c r="C30" s="67" t="s">
+        <v>353</v>
+      </c>
+      <c r="D30" s="69" t="s">
+        <v>618</v>
+      </c>
+      <c r="E30" s="70" t="s">
+        <v>402</v>
+      </c>
+      <c r="F30" s="43"/>
+      <c r="G30" s="43"/>
+    </row>
+    <row r="31" spans="1:7" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A31" s="66" t="s">
+        <v>619</v>
+      </c>
+      <c r="B31" s="38" t="s">
+        <v>620</v>
+      </c>
+      <c r="C31" s="67" t="s">
+        <v>354</v>
+      </c>
+      <c r="D31" s="38" t="s">
+        <v>621</v>
+      </c>
+      <c r="E31" s="68" t="s">
+        <v>33</v>
+      </c>
+      <c r="F31" s="43"/>
+      <c r="G31" s="43"/>
+    </row>
+    <row r="32" spans="1:7" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A32" s="66"/>
+      <c r="B32" s="38" t="s">
+        <v>622</v>
+      </c>
+      <c r="C32" s="67" t="s">
+        <v>355</v>
+      </c>
+      <c r="D32" s="38" t="s">
+        <v>623</v>
+      </c>
+      <c r="E32" s="68" t="s">
+        <v>33</v>
+      </c>
+      <c r="F32" s="43"/>
+      <c r="G32" s="43"/>
+    </row>
+    <row r="33" spans="1:7" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A33" s="66"/>
+      <c r="B33" s="38" t="s">
+        <v>624</v>
+      </c>
+      <c r="C33" s="67" t="s">
+        <v>356</v>
+      </c>
+      <c r="D33" s="38" t="s">
+        <v>625</v>
+      </c>
+      <c r="E33" s="68" t="s">
+        <v>33</v>
+      </c>
+      <c r="F33" s="43"/>
+      <c r="G33" s="43"/>
+    </row>
+    <row r="34" spans="1:7" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A34" s="66"/>
+      <c r="B34" s="38" t="s">
+        <v>626</v>
+      </c>
+      <c r="C34" s="67" t="s">
+        <v>357</v>
+      </c>
+      <c r="D34" s="38" t="s">
+        <v>627</v>
+      </c>
+      <c r="E34" s="68" t="s">
+        <v>33</v>
+      </c>
+      <c r="F34" s="43"/>
+      <c r="G34" s="43"/>
+    </row>
+    <row r="35" spans="1:7" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A35" s="66"/>
+      <c r="B35" s="38" t="s">
+        <v>628</v>
+      </c>
+      <c r="C35" s="67" t="s">
+        <v>358</v>
+      </c>
+      <c r="D35" s="38" t="s">
+        <v>629</v>
+      </c>
+      <c r="E35" s="68" t="s">
+        <v>33</v>
+      </c>
+      <c r="F35" s="43"/>
+      <c r="G35" s="43"/>
+    </row>
+    <row r="36" spans="1:7" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A36" s="66"/>
+      <c r="B36" s="69" t="s">
+        <v>630</v>
+      </c>
+      <c r="C36" s="67" t="s">
+        <v>359</v>
+      </c>
+      <c r="D36" s="69" t="s">
+        <v>631</v>
+      </c>
+      <c r="E36" s="70" t="s">
+        <v>402</v>
+      </c>
+      <c r="F36" s="43"/>
+      <c r="G36" s="43"/>
+    </row>
+    <row r="37" spans="1:7" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A37" s="66" t="s">
+        <v>632</v>
+      </c>
+      <c r="B37" s="38" t="s">
+        <v>620</v>
+      </c>
+      <c r="C37" s="67" t="s">
+        <v>360</v>
+      </c>
+      <c r="D37" s="38" t="s">
+        <v>633</v>
+      </c>
+      <c r="E37" s="68" t="s">
+        <v>33</v>
+      </c>
+      <c r="F37" s="43"/>
+      <c r="G37" s="43"/>
+    </row>
+    <row r="38" spans="1:7" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A38" s="66"/>
+      <c r="B38" s="38" t="s">
+        <v>622</v>
+      </c>
+      <c r="C38" s="67" t="s">
+        <v>361</v>
+      </c>
+      <c r="D38" s="38" t="s">
+        <v>634</v>
+      </c>
+      <c r="E38" s="68" t="s">
+        <v>33</v>
+      </c>
+      <c r="F38" s="43"/>
+      <c r="G38" s="43"/>
+    </row>
+    <row r="39" spans="1:7" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A39" s="66"/>
+      <c r="B39" s="38" t="s">
+        <v>624</v>
+      </c>
+      <c r="C39" s="67" t="s">
+        <v>362</v>
+      </c>
+      <c r="D39" s="38" t="s">
+        <v>635</v>
+      </c>
+      <c r="E39" s="68" t="s">
+        <v>33</v>
+      </c>
+      <c r="F39" s="43"/>
+      <c r="G39" s="43"/>
+    </row>
+    <row r="40" spans="1:7" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A40" s="66"/>
+      <c r="B40" s="38" t="s">
+        <v>626</v>
+      </c>
+      <c r="C40" s="67" t="s">
+        <v>363</v>
+      </c>
+      <c r="D40" s="38" t="s">
+        <v>636</v>
+      </c>
+      <c r="E40" s="68" t="s">
+        <v>33</v>
+      </c>
+      <c r="F40" s="43"/>
+      <c r="G40" s="43"/>
+    </row>
+    <row r="41" spans="1:7" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A41" s="66"/>
+      <c r="B41" s="38" t="s">
+        <v>628</v>
+      </c>
+      <c r="C41" s="67" t="s">
+        <v>364</v>
+      </c>
+      <c r="D41" s="38" t="s">
+        <v>637</v>
+      </c>
+      <c r="E41" s="68" t="s">
+        <v>33</v>
+      </c>
+      <c r="F41" s="43"/>
+      <c r="G41" s="43"/>
+    </row>
+    <row r="42" spans="1:7" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A42" s="66"/>
+      <c r="B42" s="69" t="s">
+        <v>638</v>
+      </c>
+      <c r="C42" s="67" t="s">
+        <v>365</v>
+      </c>
+      <c r="D42" s="69" t="s">
+        <v>639</v>
+      </c>
+      <c r="E42" s="70" t="s">
+        <v>402</v>
+      </c>
+      <c r="F42" s="43"/>
+      <c r="G42" s="43"/>
+    </row>
+    <row r="43" spans="1:7" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A43" s="66" t="s">
+        <v>640</v>
+      </c>
+      <c r="B43" s="38" t="s">
+        <v>620</v>
+      </c>
+      <c r="C43" s="67" t="s">
+        <v>366</v>
+      </c>
+      <c r="D43" s="38" t="s">
+        <v>641</v>
+      </c>
+      <c r="E43" s="68" t="s">
+        <v>33</v>
+      </c>
+      <c r="F43" s="43"/>
+      <c r="G43" s="43"/>
+    </row>
+    <row r="44" spans="1:7" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A44" s="66"/>
+      <c r="B44" s="38" t="s">
+        <v>622</v>
+      </c>
+      <c r="C44" s="67" t="s">
+        <v>367</v>
+      </c>
+      <c r="D44" s="38" t="s">
+        <v>642</v>
+      </c>
+      <c r="E44" s="68" t="s">
+        <v>33</v>
+      </c>
+      <c r="F44" s="43"/>
+      <c r="G44" s="43"/>
+    </row>
+    <row r="45" spans="1:7" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A45" s="66"/>
+      <c r="B45" s="38" t="s">
+        <v>624</v>
+      </c>
+      <c r="C45" s="67" t="s">
+        <v>368</v>
+      </c>
+      <c r="D45" s="38" t="s">
+        <v>643</v>
+      </c>
+      <c r="E45" s="68" t="s">
+        <v>33</v>
+      </c>
+      <c r="F45" s="43"/>
+      <c r="G45" s="43"/>
+    </row>
+    <row r="46" spans="1:7" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A46" s="66"/>
+      <c r="B46" s="38" t="s">
+        <v>626</v>
+      </c>
+      <c r="C46" s="67" t="s">
+        <v>369</v>
+      </c>
+      <c r="D46" s="38" t="s">
+        <v>644</v>
+      </c>
+      <c r="E46" s="68" t="s">
+        <v>33</v>
+      </c>
+      <c r="F46" s="43"/>
+      <c r="G46" s="43"/>
+    </row>
+    <row r="47" spans="1:7" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A47" s="66"/>
+      <c r="B47" s="38" t="s">
+        <v>628</v>
+      </c>
+      <c r="C47" s="67" t="s">
+        <v>370</v>
+      </c>
+      <c r="D47" s="38" t="s">
+        <v>645</v>
+      </c>
+      <c r="E47" s="68" t="s">
+        <v>33</v>
+      </c>
+      <c r="F47" s="43"/>
+      <c r="G47" s="43"/>
+    </row>
+    <row r="48" spans="1:7" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A48" s="66"/>
+      <c r="B48" s="69" t="s">
+        <v>646</v>
+      </c>
+      <c r="C48" s="67" t="s">
+        <v>371</v>
+      </c>
+      <c r="D48" s="69" t="s">
+        <v>647</v>
+      </c>
+      <c r="E48" s="70" t="s">
+        <v>402</v>
+      </c>
+      <c r="F48" s="43"/>
+      <c r="G48" s="43"/>
+    </row>
+    <row r="49" spans="1:7" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A49" s="66" t="s">
+        <v>648</v>
+      </c>
+      <c r="B49" s="38" t="s">
+        <v>620</v>
+      </c>
+      <c r="C49" s="67" t="s">
+        <v>372</v>
+      </c>
+      <c r="D49" s="38" t="s">
+        <v>649</v>
+      </c>
+      <c r="E49" s="68" t="s">
+        <v>33</v>
+      </c>
+      <c r="F49" s="43"/>
+      <c r="G49" s="43"/>
+    </row>
+    <row r="50" spans="1:7" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A50" s="66"/>
+      <c r="B50" s="38" t="s">
+        <v>622</v>
+      </c>
+      <c r="C50" s="67" t="s">
+        <v>373</v>
+      </c>
+      <c r="D50" s="38" t="s">
+        <v>650</v>
+      </c>
+      <c r="E50" s="68" t="s">
+        <v>33</v>
+      </c>
+      <c r="F50" s="43"/>
+      <c r="G50" s="43"/>
+    </row>
+    <row r="51" spans="1:7" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A51" s="66"/>
+      <c r="B51" s="38" t="s">
+        <v>624</v>
+      </c>
+      <c r="C51" s="67" t="s">
+        <v>374</v>
+      </c>
+      <c r="D51" s="38" t="s">
+        <v>651</v>
+      </c>
+      <c r="E51" s="68" t="s">
+        <v>33</v>
+      </c>
+      <c r="F51" s="43"/>
+      <c r="G51" s="43"/>
+    </row>
+    <row r="52" spans="1:7" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A52" s="66"/>
+      <c r="B52" s="38" t="s">
+        <v>626</v>
+      </c>
+      <c r="C52" s="67" t="s">
+        <v>375</v>
+      </c>
+      <c r="D52" s="38" t="s">
+        <v>652</v>
+      </c>
+      <c r="E52" s="68" t="s">
+        <v>33</v>
+      </c>
+      <c r="F52" s="43"/>
+      <c r="G52" s="43"/>
+    </row>
+    <row r="53" spans="1:7" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A53" s="66"/>
+      <c r="B53" s="38" t="s">
+        <v>628</v>
+      </c>
+      <c r="C53" s="67" t="s">
+        <v>376</v>
+      </c>
+      <c r="D53" s="38" t="s">
+        <v>653</v>
+      </c>
+      <c r="E53" s="68" t="s">
+        <v>33</v>
+      </c>
+      <c r="F53" s="43"/>
+      <c r="G53" s="43"/>
+    </row>
+    <row r="54" spans="1:7" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A54" s="66"/>
+      <c r="B54" s="69" t="s">
+        <v>654</v>
+      </c>
+      <c r="C54" s="67" t="s">
+        <v>377</v>
+      </c>
+      <c r="D54" s="69" t="s">
+        <v>655</v>
+      </c>
+      <c r="E54" s="70" t="s">
+        <v>402</v>
+      </c>
+      <c r="F54" s="43"/>
+      <c r="G54" s="43"/>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A55" s="43"/>
+      <c r="B55" s="43"/>
+      <c r="D55" s="43"/>
+      <c r="F55" s="43"/>
+      <c r="G55" s="43"/>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A56" s="43"/>
+      <c r="B56" s="43"/>
+      <c r="D56" s="43"/>
+      <c r="F56" s="43"/>
+      <c r="G56" s="43"/>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A57" s="43"/>
+      <c r="B57" s="43"/>
+      <c r="D57" s="43"/>
+      <c r="F57" s="43"/>
+      <c r="G57" s="43"/>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A58" s="43"/>
+      <c r="B58" s="43"/>
+      <c r="D58" s="43"/>
+      <c r="F58" s="43"/>
+      <c r="G58" s="43"/>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A59" s="43"/>
+      <c r="B59" s="43"/>
+      <c r="D59" s="43"/>
+      <c r="F59" s="43"/>
+      <c r="G59" s="43"/>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A1:A15"/>
+    <mergeCell ref="A16:A30"/>
+    <mergeCell ref="A31:A36"/>
+    <mergeCell ref="A37:A42"/>
+    <mergeCell ref="A43:A48"/>
+    <mergeCell ref="A49:A54"/>
+  </mergeCells>
+  <phoneticPr fontId="12" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D1CDA5CE-CBE3-4ABD-8EB5-73C1BE3752FD}">
+  <dimension ref="A1:E116"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="27.28515625" customWidth="1"/>
+    <col min="2" max="2" width="31.5703125" customWidth="1"/>
+    <col min="4" max="4" width="31.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A1" s="66" t="s">
+        <v>663</v>
+      </c>
+      <c r="B1" s="38" t="s">
+        <v>580</v>
+      </c>
+      <c r="C1" s="38" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="38" t="s">
+        <v>664</v>
+      </c>
+      <c r="E1" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A2" s="66"/>
+      <c r="B2" s="38" t="s">
+        <v>582</v>
+      </c>
+      <c r="C2" s="38" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="38" t="s">
+        <v>665</v>
+      </c>
+      <c r="E2" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A3" s="66"/>
+      <c r="B3" s="38" t="s">
+        <v>584</v>
+      </c>
+      <c r="C3" s="38" t="s">
+        <v>3</v>
+      </c>
+      <c r="D3" s="38" t="s">
+        <v>666</v>
+      </c>
+      <c r="E3" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A4" s="66"/>
+      <c r="B4" s="38" t="s">
+        <v>215</v>
+      </c>
+      <c r="C4" s="38" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4" s="38" t="s">
+        <v>667</v>
+      </c>
+      <c r="E4" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A5" s="66"/>
+      <c r="B5" s="38" t="s">
+        <v>216</v>
+      </c>
+      <c r="C5" s="38" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="38" t="s">
+        <v>668</v>
+      </c>
+      <c r="E5" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A6" s="66"/>
+      <c r="B6" s="38" t="s">
+        <v>669</v>
+      </c>
+      <c r="C6" s="38" t="s">
+        <v>9</v>
+      </c>
+      <c r="D6" s="38" t="s">
+        <v>670</v>
+      </c>
+      <c r="E6" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A7" s="66"/>
+      <c r="B7" s="38" t="s">
+        <v>671</v>
+      </c>
+      <c r="C7" s="38" t="s">
+        <v>12</v>
+      </c>
+      <c r="D7" s="38" t="s">
+        <v>672</v>
+      </c>
+      <c r="E7" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A8" s="66"/>
+      <c r="B8" s="38" t="s">
+        <v>673</v>
+      </c>
+      <c r="C8" s="38" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" s="38" t="s">
+        <v>674</v>
+      </c>
+      <c r="E8" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A9" s="66"/>
+      <c r="B9" s="38" t="s">
+        <v>660</v>
+      </c>
+      <c r="C9" s="38" t="s">
+        <v>16</v>
+      </c>
+      <c r="D9" s="38" t="s">
+        <v>675</v>
+      </c>
+      <c r="E9" s="70" t="s">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A10" s="66"/>
+      <c r="B10" s="38" t="s">
+        <v>661</v>
+      </c>
+      <c r="C10" s="38" t="s">
+        <v>18</v>
+      </c>
+      <c r="D10" s="38" t="s">
+        <v>676</v>
+      </c>
+      <c r="E10" s="70" t="s">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A11" s="66"/>
+      <c r="B11" s="38" t="s">
+        <v>559</v>
+      </c>
+      <c r="C11" s="38" t="s">
+        <v>19</v>
+      </c>
+      <c r="D11" s="38" t="s">
+        <v>677</v>
+      </c>
+      <c r="E11" s="70" t="s">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A12" s="66"/>
+      <c r="B12" s="38" t="s">
+        <v>564</v>
+      </c>
+      <c r="C12" s="38" t="s">
+        <v>20</v>
+      </c>
+      <c r="D12" s="38" t="s">
+        <v>678</v>
+      </c>
+      <c r="E12" s="70" t="s">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A13" s="66"/>
+      <c r="B13" s="38" t="s">
+        <v>232</v>
+      </c>
+      <c r="C13" s="38" t="s">
+        <v>21</v>
+      </c>
+      <c r="D13" s="38" t="s">
+        <v>679</v>
+      </c>
+      <c r="E13" s="76" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A14" s="66" t="s">
+        <v>680</v>
+      </c>
+      <c r="B14" s="38" t="s">
+        <v>580</v>
+      </c>
+      <c r="C14" s="38" t="s">
+        <v>22</v>
+      </c>
+      <c r="D14" s="38" t="s">
+        <v>681</v>
+      </c>
+      <c r="E14" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A15" s="66"/>
+      <c r="B15" s="38" t="s">
+        <v>582</v>
+      </c>
+      <c r="C15" s="38" t="s">
+        <v>23</v>
+      </c>
+      <c r="D15" s="38" t="s">
+        <v>682</v>
+      </c>
+      <c r="E15" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A16" s="66"/>
+      <c r="B16" s="38" t="s">
+        <v>584</v>
+      </c>
+      <c r="C16" s="38" t="s">
+        <v>24</v>
+      </c>
+      <c r="D16" s="38" t="s">
+        <v>683</v>
+      </c>
+      <c r="E16" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A17" s="66"/>
+      <c r="B17" s="38" t="s">
+        <v>215</v>
+      </c>
+      <c r="C17" s="38" t="s">
+        <v>112</v>
+      </c>
+      <c r="D17" s="38" t="s">
+        <v>684</v>
+      </c>
+      <c r="E17" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A18" s="66"/>
+      <c r="B18" s="38" t="s">
+        <v>216</v>
+      </c>
+      <c r="C18" s="38" t="s">
+        <v>113</v>
+      </c>
+      <c r="D18" s="38" t="s">
+        <v>685</v>
+      </c>
+      <c r="E18" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A19" s="66"/>
+      <c r="B19" s="38" t="s">
+        <v>669</v>
+      </c>
+      <c r="C19" s="38" t="s">
+        <v>114</v>
+      </c>
+      <c r="D19" s="38" t="s">
+        <v>686</v>
+      </c>
+      <c r="E19" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A20" s="66"/>
+      <c r="B20" s="38" t="s">
+        <v>671</v>
+      </c>
+      <c r="C20" s="38" t="s">
+        <v>115</v>
+      </c>
+      <c r="D20" s="38" t="s">
+        <v>687</v>
+      </c>
+      <c r="E20" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A21" s="66"/>
+      <c r="B21" s="38" t="s">
+        <v>673</v>
+      </c>
+      <c r="C21" s="38" t="s">
+        <v>117</v>
+      </c>
+      <c r="D21" s="38" t="s">
+        <v>688</v>
+      </c>
+      <c r="E21" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A22" s="66"/>
+      <c r="B22" s="38" t="s">
+        <v>660</v>
+      </c>
+      <c r="C22" s="38" t="s">
+        <v>119</v>
+      </c>
+      <c r="D22" s="38" t="s">
+        <v>689</v>
+      </c>
+      <c r="E22" s="70" t="s">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A23" s="66"/>
+      <c r="B23" s="38" t="s">
+        <v>661</v>
+      </c>
+      <c r="C23" s="38" t="s">
+        <v>121</v>
+      </c>
+      <c r="D23" s="38" t="s">
+        <v>690</v>
+      </c>
+      <c r="E23" s="70" t="s">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A24" s="66"/>
+      <c r="B24" s="38" t="s">
+        <v>559</v>
+      </c>
+      <c r="C24" s="38" t="s">
+        <v>123</v>
+      </c>
+      <c r="D24" s="38" t="s">
+        <v>691</v>
+      </c>
+      <c r="E24" s="70" t="s">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A25" s="66"/>
+      <c r="B25" s="38" t="s">
+        <v>564</v>
+      </c>
+      <c r="C25" s="38" t="s">
+        <v>348</v>
+      </c>
+      <c r="D25" s="38" t="s">
+        <v>692</v>
+      </c>
+      <c r="E25" s="70" t="s">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A26" s="66"/>
+      <c r="B26" s="38" t="s">
+        <v>232</v>
+      </c>
+      <c r="C26" s="38" t="s">
+        <v>349</v>
+      </c>
+      <c r="D26" s="38" t="s">
+        <v>693</v>
+      </c>
+      <c r="E26" s="76" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A27" s="66" t="s">
+        <v>694</v>
+      </c>
+      <c r="B27" s="38" t="s">
+        <v>580</v>
+      </c>
+      <c r="C27" s="38" t="s">
+        <v>350</v>
+      </c>
+      <c r="D27" s="38" t="s">
+        <v>695</v>
+      </c>
+      <c r="E27" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A28" s="66"/>
+      <c r="B28" s="38" t="s">
+        <v>582</v>
+      </c>
+      <c r="C28" s="38" t="s">
+        <v>351</v>
+      </c>
+      <c r="D28" s="38" t="s">
+        <v>696</v>
+      </c>
+      <c r="E28" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A29" s="66"/>
+      <c r="B29" s="38" t="s">
+        <v>584</v>
+      </c>
+      <c r="C29" s="38" t="s">
+        <v>352</v>
+      </c>
+      <c r="D29" s="38" t="s">
+        <v>697</v>
+      </c>
+      <c r="E29" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A30" s="66"/>
+      <c r="B30" s="38" t="s">
+        <v>215</v>
+      </c>
+      <c r="C30" s="38" t="s">
+        <v>353</v>
+      </c>
+      <c r="D30" s="38" t="s">
+        <v>698</v>
+      </c>
+      <c r="E30" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A31" s="66"/>
+      <c r="B31" s="38" t="s">
+        <v>216</v>
+      </c>
+      <c r="C31" s="38" t="s">
+        <v>354</v>
+      </c>
+      <c r="D31" s="38" t="s">
+        <v>699</v>
+      </c>
+      <c r="E31" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A32" s="66"/>
+      <c r="B32" s="38" t="s">
+        <v>669</v>
+      </c>
+      <c r="C32" s="38" t="s">
+        <v>355</v>
+      </c>
+      <c r="D32" s="38" t="s">
+        <v>700</v>
+      </c>
+      <c r="E32" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A33" s="66"/>
+      <c r="B33" s="38" t="s">
+        <v>671</v>
+      </c>
+      <c r="C33" s="38" t="s">
+        <v>356</v>
+      </c>
+      <c r="D33" s="38" t="s">
+        <v>701</v>
+      </c>
+      <c r="E33" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A34" s="66"/>
+      <c r="B34" s="38" t="s">
+        <v>673</v>
+      </c>
+      <c r="C34" s="38" t="s">
+        <v>357</v>
+      </c>
+      <c r="D34" s="38" t="s">
+        <v>702</v>
+      </c>
+      <c r="E34" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A35" s="66"/>
+      <c r="B35" s="38" t="s">
+        <v>660</v>
+      </c>
+      <c r="C35" s="38" t="s">
+        <v>358</v>
+      </c>
+      <c r="D35" s="38" t="s">
+        <v>703</v>
+      </c>
+      <c r="E35" s="70" t="s">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A36" s="66"/>
+      <c r="B36" s="38" t="s">
+        <v>661</v>
+      </c>
+      <c r="C36" s="38" t="s">
+        <v>359</v>
+      </c>
+      <c r="D36" s="38" t="s">
+        <v>704</v>
+      </c>
+      <c r="E36" s="70" t="s">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A37" s="66"/>
+      <c r="B37" s="38" t="s">
+        <v>559</v>
+      </c>
+      <c r="C37" s="38" t="s">
+        <v>360</v>
+      </c>
+      <c r="D37" s="38" t="s">
+        <v>705</v>
+      </c>
+      <c r="E37" s="70" t="s">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A38" s="66"/>
+      <c r="B38" s="38" t="s">
+        <v>564</v>
+      </c>
+      <c r="C38" s="38" t="s">
+        <v>361</v>
+      </c>
+      <c r="D38" s="38" t="s">
+        <v>706</v>
+      </c>
+      <c r="E38" s="70" t="s">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A39" s="66"/>
+      <c r="B39" s="38" t="s">
+        <v>232</v>
+      </c>
+      <c r="C39" s="38" t="s">
+        <v>362</v>
+      </c>
+      <c r="D39" s="38" t="s">
+        <v>707</v>
+      </c>
+      <c r="E39" s="76" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A40" s="66" t="s">
+        <v>708</v>
+      </c>
+      <c r="B40" s="38" t="s">
+        <v>580</v>
+      </c>
+      <c r="C40" s="38" t="s">
+        <v>363</v>
+      </c>
+      <c r="D40" s="38" t="s">
+        <v>709</v>
+      </c>
+      <c r="E40" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A41" s="66"/>
+      <c r="B41" s="38" t="s">
+        <v>582</v>
+      </c>
+      <c r="C41" s="38" t="s">
+        <v>364</v>
+      </c>
+      <c r="D41" s="38" t="s">
+        <v>710</v>
+      </c>
+      <c r="E41" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A42" s="66"/>
+      <c r="B42" s="38" t="s">
+        <v>584</v>
+      </c>
+      <c r="C42" s="38" t="s">
+        <v>365</v>
+      </c>
+      <c r="D42" s="38" t="s">
+        <v>711</v>
+      </c>
+      <c r="E42" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A43" s="66"/>
+      <c r="B43" s="38" t="s">
+        <v>215</v>
+      </c>
+      <c r="C43" s="38" t="s">
+        <v>366</v>
+      </c>
+      <c r="D43" s="38" t="s">
+        <v>712</v>
+      </c>
+      <c r="E43" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A44" s="66"/>
+      <c r="B44" s="38" t="s">
+        <v>216</v>
+      </c>
+      <c r="C44" s="38" t="s">
+        <v>367</v>
+      </c>
+      <c r="D44" s="38" t="s">
+        <v>713</v>
+      </c>
+      <c r="E44" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A45" s="66"/>
+      <c r="B45" s="38" t="s">
+        <v>669</v>
+      </c>
+      <c r="C45" s="38" t="s">
+        <v>368</v>
+      </c>
+      <c r="D45" s="38" t="s">
+        <v>714</v>
+      </c>
+      <c r="E45" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A46" s="66"/>
+      <c r="B46" s="38" t="s">
+        <v>671</v>
+      </c>
+      <c r="C46" s="38" t="s">
+        <v>369</v>
+      </c>
+      <c r="D46" s="38" t="s">
+        <v>715</v>
+      </c>
+      <c r="E46" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A47" s="66"/>
+      <c r="B47" s="38" t="s">
+        <v>673</v>
+      </c>
+      <c r="C47" s="38" t="s">
+        <v>370</v>
+      </c>
+      <c r="D47" s="38" t="s">
+        <v>716</v>
+      </c>
+      <c r="E47" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A48" s="66"/>
+      <c r="B48" s="38" t="s">
+        <v>660</v>
+      </c>
+      <c r="C48" s="38" t="s">
+        <v>371</v>
+      </c>
+      <c r="D48" s="38" t="s">
+        <v>717</v>
+      </c>
+      <c r="E48" s="70" t="s">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A49" s="66"/>
+      <c r="B49" s="38" t="s">
+        <v>661</v>
+      </c>
+      <c r="C49" s="38" t="s">
+        <v>372</v>
+      </c>
+      <c r="D49" s="38" t="s">
+        <v>718</v>
+      </c>
+      <c r="E49" s="70" t="s">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A50" s="66"/>
+      <c r="B50" s="38" t="s">
+        <v>559</v>
+      </c>
+      <c r="C50" s="38" t="s">
+        <v>373</v>
+      </c>
+      <c r="D50" s="38" t="s">
+        <v>719</v>
+      </c>
+      <c r="E50" s="70" t="s">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A51" s="66"/>
+      <c r="B51" s="38" t="s">
+        <v>564</v>
+      </c>
+      <c r="C51" s="38" t="s">
+        <v>374</v>
+      </c>
+      <c r="D51" s="38" t="s">
+        <v>720</v>
+      </c>
+      <c r="E51" s="70" t="s">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A52" s="66"/>
+      <c r="B52" s="38" t="s">
+        <v>232</v>
+      </c>
+      <c r="C52" s="38" t="s">
+        <v>375</v>
+      </c>
+      <c r="D52" s="38" t="s">
+        <v>721</v>
+      </c>
+      <c r="E52" s="76" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A53" s="66" t="s">
+        <v>786</v>
+      </c>
+      <c r="B53" s="38" t="s">
+        <v>580</v>
+      </c>
+      <c r="C53" s="38" t="s">
+        <v>376</v>
+      </c>
+      <c r="D53" s="38" t="s">
+        <v>722</v>
+      </c>
+      <c r="E53" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A54" s="66"/>
+      <c r="B54" s="38" t="s">
+        <v>582</v>
+      </c>
+      <c r="C54" s="38" t="s">
+        <v>377</v>
+      </c>
+      <c r="D54" s="38" t="s">
+        <v>723</v>
+      </c>
+      <c r="E54" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A55" s="66"/>
+      <c r="B55" s="38" t="s">
+        <v>584</v>
+      </c>
+      <c r="C55" s="38" t="s">
+        <v>378</v>
+      </c>
+      <c r="D55" s="38" t="s">
+        <v>724</v>
+      </c>
+      <c r="E55" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A56" s="66"/>
+      <c r="B56" s="38" t="s">
+        <v>215</v>
+      </c>
+      <c r="C56" s="38" t="s">
+        <v>379</v>
+      </c>
+      <c r="D56" s="38" t="s">
+        <v>725</v>
+      </c>
+      <c r="E56" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A57" s="66"/>
+      <c r="B57" s="38" t="s">
+        <v>216</v>
+      </c>
+      <c r="C57" s="38" t="s">
+        <v>380</v>
+      </c>
+      <c r="D57" s="38" t="s">
+        <v>726</v>
+      </c>
+      <c r="E57" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A58" s="66"/>
+      <c r="B58" s="38" t="s">
+        <v>669</v>
+      </c>
+      <c r="C58" s="38" t="s">
+        <v>381</v>
+      </c>
+      <c r="D58" s="38" t="s">
+        <v>727</v>
+      </c>
+      <c r="E58" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A59" s="66"/>
+      <c r="B59" s="38" t="s">
+        <v>671</v>
+      </c>
+      <c r="C59" s="38" t="s">
+        <v>382</v>
+      </c>
+      <c r="D59" s="38" t="s">
+        <v>728</v>
+      </c>
+      <c r="E59" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A60" s="66"/>
+      <c r="B60" s="38" t="s">
+        <v>232</v>
+      </c>
+      <c r="C60" s="38" t="s">
+        <v>383</v>
+      </c>
+      <c r="D60" s="38" t="s">
+        <v>729</v>
+      </c>
+      <c r="E60" s="76" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A61" s="66" t="s">
+        <v>787</v>
+      </c>
+      <c r="B61" s="38" t="s">
+        <v>580</v>
+      </c>
+      <c r="C61" s="38" t="s">
+        <v>384</v>
+      </c>
+      <c r="D61" s="38" t="s">
+        <v>730</v>
+      </c>
+      <c r="E61" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A62" s="66"/>
+      <c r="B62" s="38" t="s">
+        <v>582</v>
+      </c>
+      <c r="C62" s="38" t="s">
+        <v>385</v>
+      </c>
+      <c r="D62" s="38" t="s">
+        <v>731</v>
+      </c>
+      <c r="E62" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A63" s="66"/>
+      <c r="B63" s="38" t="s">
+        <v>584</v>
+      </c>
+      <c r="C63" s="38" t="s">
+        <v>386</v>
+      </c>
+      <c r="D63" s="38" t="s">
+        <v>732</v>
+      </c>
+      <c r="E63" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A64" s="66"/>
+      <c r="B64" s="38" t="s">
+        <v>215</v>
+      </c>
+      <c r="C64" s="38" t="s">
+        <v>387</v>
+      </c>
+      <c r="D64" s="38" t="s">
+        <v>733</v>
+      </c>
+      <c r="E64" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A65" s="66"/>
+      <c r="B65" s="38" t="s">
+        <v>216</v>
+      </c>
+      <c r="C65" s="38" t="s">
+        <v>388</v>
+      </c>
+      <c r="D65" s="38" t="s">
+        <v>734</v>
+      </c>
+      <c r="E65" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A66" s="66"/>
+      <c r="B66" s="38" t="s">
+        <v>669</v>
+      </c>
+      <c r="C66" s="38" t="s">
+        <v>389</v>
+      </c>
+      <c r="D66" s="38" t="s">
+        <v>735</v>
+      </c>
+      <c r="E66" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A67" s="66"/>
+      <c r="B67" s="38" t="s">
+        <v>671</v>
+      </c>
+      <c r="C67" s="38" t="s">
+        <v>390</v>
+      </c>
+      <c r="D67" s="38" t="s">
+        <v>736</v>
+      </c>
+      <c r="E67" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A68" s="66"/>
+      <c r="B68" s="38" t="s">
+        <v>232</v>
+      </c>
+      <c r="C68" s="38" t="s">
+        <v>391</v>
+      </c>
+      <c r="D68" s="38" t="s">
+        <v>737</v>
+      </c>
+      <c r="E68" s="76" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A69" s="66" t="s">
+        <v>788</v>
+      </c>
+      <c r="B69" s="38" t="s">
+        <v>580</v>
+      </c>
+      <c r="C69" s="38" t="s">
+        <v>392</v>
+      </c>
+      <c r="D69" s="38" t="s">
+        <v>738</v>
+      </c>
+      <c r="E69" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A70" s="66"/>
+      <c r="B70" s="38" t="s">
+        <v>582</v>
+      </c>
+      <c r="C70" s="38" t="s">
+        <v>393</v>
+      </c>
+      <c r="D70" s="38" t="s">
+        <v>739</v>
+      </c>
+      <c r="E70" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A71" s="66"/>
+      <c r="B71" s="38" t="s">
+        <v>584</v>
+      </c>
+      <c r="C71" s="38" t="s">
+        <v>394</v>
+      </c>
+      <c r="D71" s="38" t="s">
+        <v>740</v>
+      </c>
+      <c r="E71" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A72" s="66"/>
+      <c r="B72" s="38" t="s">
+        <v>215</v>
+      </c>
+      <c r="C72" s="38" t="s">
+        <v>395</v>
+      </c>
+      <c r="D72" s="38" t="s">
+        <v>741</v>
+      </c>
+      <c r="E72" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A73" s="66"/>
+      <c r="B73" s="38" t="s">
+        <v>216</v>
+      </c>
+      <c r="C73" s="38" t="s">
+        <v>396</v>
+      </c>
+      <c r="D73" s="38" t="s">
+        <v>742</v>
+      </c>
+      <c r="E73" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A74" s="66"/>
+      <c r="B74" s="38" t="s">
+        <v>669</v>
+      </c>
+      <c r="C74" s="38" t="s">
+        <v>397</v>
+      </c>
+      <c r="D74" s="38" t="s">
+        <v>743</v>
+      </c>
+      <c r="E74" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A75" s="66"/>
+      <c r="B75" s="38" t="s">
+        <v>671</v>
+      </c>
+      <c r="C75" s="38" t="s">
+        <v>398</v>
+      </c>
+      <c r="D75" s="38" t="s">
+        <v>744</v>
+      </c>
+      <c r="E75" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A76" s="66"/>
+      <c r="B76" s="38" t="s">
+        <v>232</v>
+      </c>
+      <c r="C76" s="38" t="s">
+        <v>399</v>
+      </c>
+      <c r="D76" s="38" t="s">
+        <v>745</v>
+      </c>
+      <c r="E76" s="76" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A77" s="66" t="s">
+        <v>789</v>
+      </c>
+      <c r="B77" s="38" t="s">
+        <v>580</v>
+      </c>
+      <c r="C77" s="38" t="s">
+        <v>400</v>
+      </c>
+      <c r="D77" s="38" t="s">
+        <v>746</v>
+      </c>
+      <c r="E77" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A78" s="66"/>
+      <c r="B78" s="38" t="s">
+        <v>582</v>
+      </c>
+      <c r="C78" s="38" t="s">
+        <v>401</v>
+      </c>
+      <c r="D78" s="38" t="s">
+        <v>747</v>
+      </c>
+      <c r="E78" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A79" s="66"/>
+      <c r="B79" s="38" t="s">
+        <v>584</v>
+      </c>
+      <c r="C79" s="38" t="s">
+        <v>794</v>
+      </c>
+      <c r="D79" s="38" t="s">
+        <v>748</v>
+      </c>
+      <c r="E79" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A80" s="66"/>
+      <c r="B80" s="38" t="s">
+        <v>215</v>
+      </c>
+      <c r="C80" s="38" t="s">
+        <v>795</v>
+      </c>
+      <c r="D80" s="38" t="s">
+        <v>749</v>
+      </c>
+      <c r="E80" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A81" s="66"/>
+      <c r="B81" s="38" t="s">
+        <v>216</v>
+      </c>
+      <c r="C81" s="38" t="s">
+        <v>796</v>
+      </c>
+      <c r="D81" s="38" t="s">
+        <v>750</v>
+      </c>
+      <c r="E81" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A82" s="66"/>
+      <c r="B82" s="38" t="s">
+        <v>669</v>
+      </c>
+      <c r="C82" s="38" t="s">
+        <v>797</v>
+      </c>
+      <c r="D82" s="38" t="s">
+        <v>751</v>
+      </c>
+      <c r="E82" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A83" s="66"/>
+      <c r="B83" s="38" t="s">
+        <v>671</v>
+      </c>
+      <c r="C83" s="38" t="s">
+        <v>798</v>
+      </c>
+      <c r="D83" s="38" t="s">
+        <v>752</v>
+      </c>
+      <c r="E83" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A84" s="66"/>
+      <c r="B84" s="38" t="s">
+        <v>232</v>
+      </c>
+      <c r="C84" s="38" t="s">
+        <v>799</v>
+      </c>
+      <c r="D84" s="38" t="s">
+        <v>753</v>
+      </c>
+      <c r="E84" s="76" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A85" s="66" t="s">
+        <v>790</v>
+      </c>
+      <c r="B85" s="38" t="s">
+        <v>580</v>
+      </c>
+      <c r="C85" s="38" t="s">
+        <v>800</v>
+      </c>
+      <c r="D85" s="38" t="s">
+        <v>754</v>
+      </c>
+      <c r="E85" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A86" s="66"/>
+      <c r="B86" s="38" t="s">
+        <v>582</v>
+      </c>
+      <c r="C86" s="38" t="s">
+        <v>801</v>
+      </c>
+      <c r="D86" s="38" t="s">
+        <v>755</v>
+      </c>
+      <c r="E86" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A87" s="66"/>
+      <c r="B87" s="38" t="s">
+        <v>584</v>
+      </c>
+      <c r="C87" s="38" t="s">
+        <v>802</v>
+      </c>
+      <c r="D87" s="38" t="s">
+        <v>756</v>
+      </c>
+      <c r="E87" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A88" s="66"/>
+      <c r="B88" s="38" t="s">
+        <v>215</v>
+      </c>
+      <c r="C88" s="38" t="s">
+        <v>803</v>
+      </c>
+      <c r="D88" s="38" t="s">
+        <v>757</v>
+      </c>
+      <c r="E88" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A89" s="66"/>
+      <c r="B89" s="38" t="s">
+        <v>216</v>
+      </c>
+      <c r="C89" s="38" t="s">
+        <v>804</v>
+      </c>
+      <c r="D89" s="38" t="s">
+        <v>758</v>
+      </c>
+      <c r="E89" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A90" s="66"/>
+      <c r="B90" s="38" t="s">
+        <v>669</v>
+      </c>
+      <c r="C90" s="38" t="s">
+        <v>805</v>
+      </c>
+      <c r="D90" s="38" t="s">
+        <v>759</v>
+      </c>
+      <c r="E90" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A91" s="66"/>
+      <c r="B91" s="38" t="s">
+        <v>671</v>
+      </c>
+      <c r="C91" s="38" t="s">
+        <v>806</v>
+      </c>
+      <c r="D91" s="38" t="s">
+        <v>760</v>
+      </c>
+      <c r="E91" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A92" s="66"/>
+      <c r="B92" s="38" t="s">
+        <v>232</v>
+      </c>
+      <c r="C92" s="38" t="s">
+        <v>807</v>
+      </c>
+      <c r="D92" s="38" t="s">
+        <v>761</v>
+      </c>
+      <c r="E92" s="76" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A93" s="66" t="s">
+        <v>791</v>
+      </c>
+      <c r="B93" s="38" t="s">
+        <v>580</v>
+      </c>
+      <c r="C93" s="38" t="s">
+        <v>808</v>
+      </c>
+      <c r="D93" s="38" t="s">
+        <v>762</v>
+      </c>
+      <c r="E93" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="94" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A94" s="66"/>
+      <c r="B94" s="38" t="s">
+        <v>582</v>
+      </c>
+      <c r="C94" s="38" t="s">
+        <v>809</v>
+      </c>
+      <c r="D94" s="38" t="s">
+        <v>763</v>
+      </c>
+      <c r="E94" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A95" s="66"/>
+      <c r="B95" s="38" t="s">
+        <v>584</v>
+      </c>
+      <c r="C95" s="38" t="s">
+        <v>810</v>
+      </c>
+      <c r="D95" s="38" t="s">
+        <v>764</v>
+      </c>
+      <c r="E95" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="96" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A96" s="66"/>
+      <c r="B96" s="38" t="s">
+        <v>215</v>
+      </c>
+      <c r="C96" s="38" t="s">
+        <v>811</v>
+      </c>
+      <c r="D96" s="38" t="s">
+        <v>765</v>
+      </c>
+      <c r="E96" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="97" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A97" s="66"/>
+      <c r="B97" s="38" t="s">
+        <v>216</v>
+      </c>
+      <c r="C97" s="38" t="s">
+        <v>812</v>
+      </c>
+      <c r="D97" s="38" t="s">
+        <v>766</v>
+      </c>
+      <c r="E97" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="98" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A98" s="66"/>
+      <c r="B98" s="38" t="s">
+        <v>669</v>
+      </c>
+      <c r="C98" s="38" t="s">
+        <v>813</v>
+      </c>
+      <c r="D98" s="38" t="s">
+        <v>767</v>
+      </c>
+      <c r="E98" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A99" s="66"/>
+      <c r="B99" s="38" t="s">
+        <v>671</v>
+      </c>
+      <c r="C99" s="38" t="s">
+        <v>814</v>
+      </c>
+      <c r="D99" s="38" t="s">
+        <v>768</v>
+      </c>
+      <c r="E99" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="100" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A100" s="66"/>
+      <c r="B100" s="38" t="s">
+        <v>232</v>
+      </c>
+      <c r="C100" s="38" t="s">
+        <v>815</v>
+      </c>
+      <c r="D100" s="38" t="s">
+        <v>769</v>
+      </c>
+      <c r="E100" s="76" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="101" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A101" s="66" t="s">
+        <v>792</v>
+      </c>
+      <c r="B101" s="38" t="s">
+        <v>580</v>
+      </c>
+      <c r="C101" s="38" t="s">
+        <v>816</v>
+      </c>
+      <c r="D101" s="38" t="s">
+        <v>770</v>
+      </c>
+      <c r="E101" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="102" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A102" s="66"/>
+      <c r="B102" s="38" t="s">
+        <v>582</v>
+      </c>
+      <c r="C102" s="38" t="s">
+        <v>817</v>
+      </c>
+      <c r="D102" s="38" t="s">
+        <v>771</v>
+      </c>
+      <c r="E102" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="103" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A103" s="66"/>
+      <c r="B103" s="38" t="s">
+        <v>584</v>
+      </c>
+      <c r="C103" s="38" t="s">
+        <v>818</v>
+      </c>
+      <c r="D103" s="38" t="s">
+        <v>772</v>
+      </c>
+      <c r="E103" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="104" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A104" s="66"/>
+      <c r="B104" s="38" t="s">
+        <v>215</v>
+      </c>
+      <c r="C104" s="38" t="s">
+        <v>819</v>
+      </c>
+      <c r="D104" s="38" t="s">
+        <v>773</v>
+      </c>
+      <c r="E104" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="105" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A105" s="66"/>
+      <c r="B105" s="38" t="s">
+        <v>216</v>
+      </c>
+      <c r="C105" s="38" t="s">
+        <v>820</v>
+      </c>
+      <c r="D105" s="38" t="s">
+        <v>774</v>
+      </c>
+      <c r="E105" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="106" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A106" s="66"/>
+      <c r="B106" s="38" t="s">
+        <v>669</v>
+      </c>
+      <c r="C106" s="38" t="s">
+        <v>821</v>
+      </c>
+      <c r="D106" s="38" t="s">
+        <v>775</v>
+      </c>
+      <c r="E106" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="107" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A107" s="66"/>
+      <c r="B107" s="38" t="s">
+        <v>671</v>
+      </c>
+      <c r="C107" s="38" t="s">
+        <v>822</v>
+      </c>
+      <c r="D107" s="38" t="s">
+        <v>776</v>
+      </c>
+      <c r="E107" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="108" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A108" s="66"/>
+      <c r="B108" s="38" t="s">
+        <v>232</v>
+      </c>
+      <c r="C108" s="38" t="s">
+        <v>823</v>
+      </c>
+      <c r="D108" s="38" t="s">
+        <v>777</v>
+      </c>
+      <c r="E108" s="76" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="109" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A109" s="66" t="s">
+        <v>793</v>
+      </c>
+      <c r="B109" s="38" t="s">
+        <v>580</v>
+      </c>
+      <c r="C109" s="38" t="s">
+        <v>824</v>
+      </c>
+      <c r="D109" s="38" t="s">
+        <v>778</v>
+      </c>
+      <c r="E109" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="110" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A110" s="66"/>
+      <c r="B110" s="38" t="s">
+        <v>582</v>
+      </c>
+      <c r="C110" s="38" t="s">
+        <v>825</v>
+      </c>
+      <c r="D110" s="38" t="s">
+        <v>779</v>
+      </c>
+      <c r="E110" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="111" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A111" s="66"/>
+      <c r="B111" s="38" t="s">
+        <v>584</v>
+      </c>
+      <c r="C111" s="38" t="s">
+        <v>826</v>
+      </c>
+      <c r="D111" s="38" t="s">
+        <v>780</v>
+      </c>
+      <c r="E111" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="112" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A112" s="66"/>
+      <c r="B112" s="38" t="s">
+        <v>215</v>
+      </c>
+      <c r="C112" s="38" t="s">
+        <v>827</v>
+      </c>
+      <c r="D112" s="38" t="s">
+        <v>781</v>
+      </c>
+      <c r="E112" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="113" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A113" s="66"/>
+      <c r="B113" s="38" t="s">
+        <v>216</v>
+      </c>
+      <c r="C113" s="38" t="s">
+        <v>828</v>
+      </c>
+      <c r="D113" s="38" t="s">
+        <v>782</v>
+      </c>
+      <c r="E113" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="114" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A114" s="66"/>
+      <c r="B114" s="38" t="s">
+        <v>669</v>
+      </c>
+      <c r="C114" s="38" t="s">
+        <v>829</v>
+      </c>
+      <c r="D114" s="38" t="s">
+        <v>783</v>
+      </c>
+      <c r="E114" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="115" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A115" s="66"/>
+      <c r="B115" s="38" t="s">
+        <v>671</v>
+      </c>
+      <c r="C115" s="38" t="s">
+        <v>830</v>
+      </c>
+      <c r="D115" s="38" t="s">
+        <v>784</v>
+      </c>
+      <c r="E115" s="70" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="116" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A116" s="66"/>
+      <c r="B116" s="38" t="s">
+        <v>232</v>
+      </c>
+      <c r="C116" s="38" t="s">
+        <v>831</v>
+      </c>
+      <c r="D116" s="38" t="s">
+        <v>785</v>
+      </c>
+      <c r="E116" s="76" t="s">
+        <v>402</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="12">
+    <mergeCell ref="A69:A76"/>
+    <mergeCell ref="A77:A84"/>
+    <mergeCell ref="A85:A92"/>
+    <mergeCell ref="A93:A100"/>
+    <mergeCell ref="A101:A108"/>
+    <mergeCell ref="A109:A116"/>
+    <mergeCell ref="A1:A13"/>
+    <mergeCell ref="A14:A26"/>
+    <mergeCell ref="A27:A39"/>
+    <mergeCell ref="A40:A52"/>
+    <mergeCell ref="A53:A60"/>
+    <mergeCell ref="A61:A68"/>
+  </mergeCells>
+  <phoneticPr fontId="12" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:I16"/>
@@ -10214,21 +13898,239 @@
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="B1:D1"/>
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="B10:D10"/>
     <mergeCell ref="B11:D11"/>
     <mergeCell ref="B12:D12"/>
     <mergeCell ref="B13:D13"/>
     <mergeCell ref="B14:D14"/>
     <mergeCell ref="B15:D15"/>
-    <mergeCell ref="B6:D6"/>
-    <mergeCell ref="B7:D7"/>
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="B9:D9"/>
-    <mergeCell ref="B10:D10"/>
-    <mergeCell ref="B1:D1"/>
-    <mergeCell ref="B2:D2"/>
-    <mergeCell ref="B3:D3"/>
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="B5:D5"/>
+  </mergeCells>
+  <phoneticPr fontId="12" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{94D4EEC2-142F-41CB-A210-C24A85D41A6F}">
+  <dimension ref="A1:E13"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="12.5703125" customWidth="1"/>
+    <col min="2" max="2" width="36.85546875" customWidth="1"/>
+    <col min="3" max="3" width="24.5703125" customWidth="1"/>
+    <col min="4" max="4" width="18.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A1" s="71" t="s">
+        <v>848</v>
+      </c>
+      <c r="B1" s="72" t="s">
+        <v>832</v>
+      </c>
+      <c r="C1" s="67" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="38" t="s">
+        <v>833</v>
+      </c>
+      <c r="E1" s="73" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A2" s="71"/>
+      <c r="B2" s="72" t="s">
+        <v>834</v>
+      </c>
+      <c r="C2" s="67" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="38" t="s">
+        <v>835</v>
+      </c>
+      <c r="E2" s="73" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A3" s="71"/>
+      <c r="B3" s="72" t="s">
+        <v>836</v>
+      </c>
+      <c r="C3" s="67" t="s">
+        <v>3</v>
+      </c>
+      <c r="D3" s="38" t="s">
+        <v>837</v>
+      </c>
+      <c r="E3" s="73" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A4" s="71"/>
+      <c r="B4" s="72" t="s">
+        <v>850</v>
+      </c>
+      <c r="C4" s="67" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4" s="38" t="s">
+        <v>838</v>
+      </c>
+      <c r="E4" s="75" t="s">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A5" s="71"/>
+      <c r="B5" s="72" t="s">
+        <v>850</v>
+      </c>
+      <c r="C5" s="67" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="38" t="s">
+        <v>839</v>
+      </c>
+      <c r="E5" s="74" t="s">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A6" s="71"/>
+      <c r="B6" s="38" t="s">
+        <v>852</v>
+      </c>
+      <c r="C6" s="67" t="s">
+        <v>9</v>
+      </c>
+      <c r="D6" s="38" t="s">
+        <v>840</v>
+      </c>
+      <c r="E6" s="73" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A7" s="71"/>
+      <c r="B7" s="38" t="s">
+        <v>853</v>
+      </c>
+      <c r="C7" s="67" t="s">
+        <v>12</v>
+      </c>
+      <c r="D7" s="38" t="s">
+        <v>841</v>
+      </c>
+      <c r="E7" s="73" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A8" s="71"/>
+      <c r="B8" s="38" t="s">
+        <v>854</v>
+      </c>
+      <c r="C8" s="67" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" s="38" t="s">
+        <v>842</v>
+      </c>
+      <c r="E8" s="73" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A9" s="71"/>
+      <c r="B9" s="38" t="s">
+        <v>855</v>
+      </c>
+      <c r="C9" s="67" t="s">
+        <v>16</v>
+      </c>
+      <c r="D9" s="38" t="s">
+        <v>843</v>
+      </c>
+      <c r="E9" s="73" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A10" s="71"/>
+      <c r="B10" s="38" t="s">
+        <v>856</v>
+      </c>
+      <c r="C10" s="67" t="s">
+        <v>18</v>
+      </c>
+      <c r="D10" s="38" t="s">
+        <v>844</v>
+      </c>
+      <c r="E10" s="73" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A11" s="71"/>
+      <c r="B11" s="38" t="s">
+        <v>857</v>
+      </c>
+      <c r="C11" s="67" t="s">
+        <v>19</v>
+      </c>
+      <c r="D11" s="38" t="s">
+        <v>845</v>
+      </c>
+      <c r="E11" s="73" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A12" s="71"/>
+      <c r="B12" s="38" t="s">
+        <v>858</v>
+      </c>
+      <c r="C12" s="67" t="s">
+        <v>20</v>
+      </c>
+      <c r="D12" s="38" t="s">
+        <v>846</v>
+      </c>
+      <c r="E12" s="73" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A13" s="71"/>
+      <c r="B13" s="38" t="s">
+        <v>859</v>
+      </c>
+      <c r="C13" s="67" t="s">
+        <v>21</v>
+      </c>
+      <c r="D13" s="38" t="s">
+        <v>847</v>
+      </c>
+      <c r="E13" s="73" t="s">
+        <v>33</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:A13"/>
   </mergeCells>
   <phoneticPr fontId="12" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -10664,22 +14566,22 @@
     </row>
   </sheetData>
   <mergeCells count="16">
-    <mergeCell ref="B1:D1"/>
-    <mergeCell ref="B2:D2"/>
-    <mergeCell ref="B3:D3"/>
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="B5:D5"/>
-    <mergeCell ref="B6:D6"/>
-    <mergeCell ref="B7:D7"/>
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="B9:D9"/>
-    <mergeCell ref="B10:D10"/>
     <mergeCell ref="B16:D16"/>
     <mergeCell ref="B11:D11"/>
     <mergeCell ref="B12:D12"/>
     <mergeCell ref="B13:D13"/>
     <mergeCell ref="B14:D14"/>
     <mergeCell ref="B15:D15"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="B10:D10"/>
+    <mergeCell ref="B1:D1"/>
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="B5:D5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -11313,16 +15215,6 @@
     </row>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="B6:D6"/>
-    <mergeCell ref="B7:D7"/>
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="B14:D14"/>
-    <mergeCell ref="B15:D15"/>
-    <mergeCell ref="B1:D1"/>
-    <mergeCell ref="B2:D2"/>
-    <mergeCell ref="B3:D3"/>
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="B5:D5"/>
     <mergeCell ref="B22:D22"/>
     <mergeCell ref="B23:D23"/>
     <mergeCell ref="B24:D24"/>
@@ -11337,6 +15229,16 @@
     <mergeCell ref="B19:D19"/>
     <mergeCell ref="B20:D20"/>
     <mergeCell ref="B21:D21"/>
+    <mergeCell ref="B1:D1"/>
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="B14:D14"/>
+    <mergeCell ref="B15:D15"/>
   </mergeCells>
   <phoneticPr fontId="12" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -11718,6 +15620,11 @@
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="B1:D1"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="B5:D5"/>
     <mergeCell ref="B11:D11"/>
     <mergeCell ref="B12:D12"/>
     <mergeCell ref="B13:D13"/>
@@ -11727,11 +15634,6 @@
     <mergeCell ref="B8:D8"/>
     <mergeCell ref="B9:D9"/>
     <mergeCell ref="B10:D10"/>
-    <mergeCell ref="B2:D2"/>
-    <mergeCell ref="B1:D1"/>
-    <mergeCell ref="B3:D3"/>
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="B5:D5"/>
   </mergeCells>
   <phoneticPr fontId="12" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -11754,11 +15656,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="59" t="s">
+      <c r="A1" s="58" t="s">
         <v>455</v>
       </c>
-      <c r="B1" s="59"/>
-      <c r="C1" s="59"/>
+      <c r="B1" s="58"/>
+      <c r="C1" s="58"/>
       <c r="D1" s="32" t="s">
         <v>0</v>
       </c>
@@ -11776,11 +15678,11 @@
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A2" s="59" t="s">
+      <c r="A2" s="58" t="s">
         <v>446</v>
       </c>
-      <c r="B2" s="59"/>
-      <c r="C2" s="59"/>
+      <c r="B2" s="58"/>
+      <c r="C2" s="58"/>
       <c r="D2" s="32" t="s">
         <v>1</v>
       </c>
@@ -11798,11 +15700,11 @@
       </c>
     </row>
     <row r="3" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="59" t="s">
+      <c r="A3" s="58" t="s">
         <v>451</v>
       </c>
-      <c r="B3" s="59"/>
-      <c r="C3" s="59"/>
+      <c r="B3" s="58"/>
+      <c r="C3" s="58"/>
       <c r="D3" s="32" t="s">
         <v>3</v>
       </c>
@@ -11820,11 +15722,11 @@
       </c>
     </row>
     <row r="4" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A4" s="59" t="s">
+      <c r="A4" s="58" t="s">
         <v>452</v>
       </c>
-      <c r="B4" s="59"/>
-      <c r="C4" s="59"/>
+      <c r="B4" s="58"/>
+      <c r="C4" s="58"/>
       <c r="D4" s="32" t="s">
         <v>5</v>
       </c>
@@ -11842,11 +15744,11 @@
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" s="59" t="s">
+      <c r="A5" s="58" t="s">
         <v>486</v>
       </c>
-      <c r="B5" s="59"/>
-      <c r="C5" s="59"/>
+      <c r="B5" s="58"/>
+      <c r="C5" s="58"/>
       <c r="D5" s="32" t="s">
         <v>7</v>
       </c>
@@ -11864,11 +15766,11 @@
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A6" s="59" t="s">
+      <c r="A6" s="58" t="s">
         <v>487</v>
       </c>
-      <c r="B6" s="59"/>
-      <c r="C6" s="59"/>
+      <c r="B6" s="58"/>
+      <c r="C6" s="58"/>
       <c r="D6" s="32" t="s">
         <v>9</v>
       </c>
@@ -11886,11 +15788,11 @@
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A7" s="58" t="s">
+      <c r="A7" s="59" t="s">
         <v>488</v>
       </c>
-      <c r="B7" s="58"/>
-      <c r="C7" s="58"/>
+      <c r="B7" s="59"/>
+      <c r="C7" s="59"/>
       <c r="D7" s="32" t="s">
         <v>12</v>
       </c>
@@ -11908,11 +15810,11 @@
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" s="58" t="s">
+      <c r="A8" s="59" t="s">
         <v>489</v>
       </c>
-      <c r="B8" s="58"/>
-      <c r="C8" s="58"/>
+      <c r="B8" s="59"/>
+      <c r="C8" s="59"/>
       <c r="D8" s="32" t="s">
         <v>14</v>
       </c>
@@ -11930,11 +15832,11 @@
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" s="58" t="s">
+      <c r="A9" s="59" t="s">
         <v>490</v>
       </c>
-      <c r="B9" s="58"/>
-      <c r="C9" s="58"/>
+      <c r="B9" s="59"/>
+      <c r="C9" s="59"/>
       <c r="D9" s="32" t="s">
         <v>16</v>
       </c>
@@ -11952,11 +15854,11 @@
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" s="58" t="s">
+      <c r="A10" s="59" t="s">
         <v>491</v>
       </c>
-      <c r="B10" s="58"/>
-      <c r="C10" s="58"/>
+      <c r="B10" s="59"/>
+      <c r="C10" s="59"/>
       <c r="D10" s="32" t="s">
         <v>18</v>
       </c>
@@ -11983,16 +15885,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="A9:C9"/>
+    <mergeCell ref="A10:C10"/>
+    <mergeCell ref="A8:C8"/>
+    <mergeCell ref="A7:C7"/>
+    <mergeCell ref="A6:C6"/>
     <mergeCell ref="A5:C5"/>
     <mergeCell ref="A4:C4"/>
     <mergeCell ref="A3:C3"/>
     <mergeCell ref="A2:C2"/>
     <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A9:C9"/>
-    <mergeCell ref="A10:C10"/>
-    <mergeCell ref="A8:C8"/>
-    <mergeCell ref="A7:C7"/>
-    <mergeCell ref="A6:C6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -12012,11 +15914,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="59" t="s">
+      <c r="A1" s="58" t="s">
         <v>455</v>
       </c>
-      <c r="B1" s="59"/>
-      <c r="C1" s="59"/>
+      <c r="B1" s="58"/>
+      <c r="C1" s="58"/>
       <c r="D1" s="32" t="s">
         <v>0</v>
       </c>
@@ -12034,11 +15936,11 @@
       </c>
     </row>
     <row r="2" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="59" t="s">
+      <c r="A2" s="58" t="s">
         <v>446</v>
       </c>
-      <c r="B2" s="59"/>
-      <c r="C2" s="59"/>
+      <c r="B2" s="58"/>
+      <c r="C2" s="58"/>
       <c r="D2" s="32" t="s">
         <v>1</v>
       </c>
@@ -12056,11 +15958,11 @@
       </c>
     </row>
     <row r="3" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="59" t="s">
+      <c r="A3" s="58" t="s">
         <v>451</v>
       </c>
-      <c r="B3" s="59"/>
-      <c r="C3" s="59"/>
+      <c r="B3" s="58"/>
+      <c r="C3" s="58"/>
       <c r="D3" s="32" t="s">
         <v>3</v>
       </c>
@@ -12078,11 +15980,11 @@
       </c>
     </row>
     <row r="4" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A4" s="59" t="s">
+      <c r="A4" s="58" t="s">
         <v>452</v>
       </c>
-      <c r="B4" s="59"/>
-      <c r="C4" s="59"/>
+      <c r="B4" s="58"/>
+      <c r="C4" s="58"/>
       <c r="D4" s="32" t="s">
         <v>5</v>
       </c>
@@ -12100,11 +16002,11 @@
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" s="59" t="s">
+      <c r="A5" s="58" t="s">
         <v>486</v>
       </c>
-      <c r="B5" s="59"/>
-      <c r="C5" s="59"/>
+      <c r="B5" s="58"/>
+      <c r="C5" s="58"/>
       <c r="D5" s="32" t="s">
         <v>7</v>
       </c>
@@ -12122,11 +16024,11 @@
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" s="59" t="s">
+      <c r="A6" s="58" t="s">
         <v>487</v>
       </c>
-      <c r="B6" s="59"/>
-      <c r="C6" s="59"/>
+      <c r="B6" s="58"/>
+      <c r="C6" s="58"/>
       <c r="D6" s="32" t="s">
         <v>9</v>
       </c>
@@ -12145,11 +16047,11 @@
       <c r="I6" s="8"/>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7" s="58" t="s">
+      <c r="A7" s="59" t="s">
         <v>488</v>
       </c>
-      <c r="B7" s="58"/>
-      <c r="C7" s="58"/>
+      <c r="B7" s="59"/>
+      <c r="C7" s="59"/>
       <c r="D7" s="32" t="s">
         <v>12</v>
       </c>
@@ -12167,11 +16069,11 @@
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" s="58" t="s">
+      <c r="A8" s="59" t="s">
         <v>489</v>
       </c>
-      <c r="B8" s="58"/>
-      <c r="C8" s="58"/>
+      <c r="B8" s="59"/>
+      <c r="C8" s="59"/>
       <c r="D8" s="32" t="s">
         <v>14</v>
       </c>
@@ -12189,11 +16091,11 @@
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9" s="58" t="s">
+      <c r="A9" s="59" t="s">
         <v>490</v>
       </c>
-      <c r="B9" s="58"/>
-      <c r="C9" s="58"/>
+      <c r="B9" s="59"/>
+      <c r="C9" s="59"/>
       <c r="D9" s="32" t="s">
         <v>16</v>
       </c>
@@ -12211,11 +16113,11 @@
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A10" s="58" t="s">
+      <c r="A10" s="59" t="s">
         <v>491</v>
       </c>
-      <c r="B10" s="58"/>
-      <c r="C10" s="58"/>
+      <c r="B10" s="59"/>
+      <c r="C10" s="59"/>
       <c r="D10" s="32" t="s">
         <v>18</v>
       </c>
@@ -12940,13 +16842,6 @@
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="A10:C10"/>
-    <mergeCell ref="A9:C9"/>
-    <mergeCell ref="A15:C15"/>
-    <mergeCell ref="A14:C14"/>
-    <mergeCell ref="A13:C13"/>
-    <mergeCell ref="A12:C12"/>
-    <mergeCell ref="A11:C11"/>
     <mergeCell ref="A3:C3"/>
     <mergeCell ref="A2:C2"/>
     <mergeCell ref="A1:C1"/>
@@ -12955,6 +16850,13 @@
     <mergeCell ref="A6:C6"/>
     <mergeCell ref="A5:C5"/>
     <mergeCell ref="A4:C4"/>
+    <mergeCell ref="A10:C10"/>
+    <mergeCell ref="A9:C9"/>
+    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="A14:C14"/>
+    <mergeCell ref="A13:C13"/>
+    <mergeCell ref="A12:C12"/>
+    <mergeCell ref="A11:C11"/>
   </mergeCells>
   <phoneticPr fontId="12" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>